<commit_message>
Separate profession selection from stat allocation screen
</commit_message>
<xml_diff>
--- a/content/game-texts.xlsx
+++ b/content/game-texts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2132" uniqueCount="807">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2153" uniqueCount="814">
   <si>
     <t>이매망량의 주인 — 산군 / 게임 텍스트 관리</t>
   </si>
@@ -2459,6 +2459,27 @@
   </si>
   <si>
     <t>직업을 바꿔도 추가 분배는 유지됩니다. 게임 시작 후에는 분배를 변경할 수 없습니다.</t>
+  </si>
+  <si>
+    <t>button.next_stats</t>
+  </si>
+  <si>
+    <t>App.tsx</t>
+  </si>
+  <si>
+    <t>다음: 스탯 분배</t>
+  </si>
+  <si>
+    <t>button.back_to_class</t>
+  </si>
+  <si>
+    <t>직업 선택으로 돌아가기</t>
+  </si>
+  <si>
+    <t>creation.allocation_step</t>
+  </si>
+  <si>
+    <t>CHARACTER / 스탯 분배</t>
   </si>
 </sst>
 </file>
@@ -2952,7 +2973,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G303"/>
+  <dimension ref="A1:G306"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -9932,8 +9953,77 @@
         <v>22</v>
       </c>
     </row>
+    <row r="304" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A304" s="5" t="s">
+        <v>807</v>
+      </c>
+      <c r="B304" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="C304" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="D304" s="6" t="s">
+        <v>809</v>
+      </c>
+      <c r="E304" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F304" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G304" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="305" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A305" s="5" t="s">
+        <v>810</v>
+      </c>
+      <c r="B305" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="C305" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="D305" s="6" t="s">
+        <v>811</v>
+      </c>
+      <c r="E305" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F305" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G305" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="306" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A306" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="B306" s="5" t="s">
+        <v>780</v>
+      </c>
+      <c r="C306" s="5" t="s">
+        <v>808</v>
+      </c>
+      <c r="D306" s="6" t="s">
+        <v>813</v>
+      </c>
+      <c r="E306" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F306" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G306" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G303"/>
+  <autoFilter ref="A1:G306"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Add victory XP progression with a level 30 cap and experience meter
</commit_message>
<xml_diff>
--- a/content/game-texts.xlsx
+++ b/content/game-texts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2153" uniqueCount="814">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2188" uniqueCount="830">
   <si>
     <t>이매망량의 주인 — 산군 / 게임 텍스트 관리</t>
   </si>
@@ -2480,6 +2480,54 @@
   </si>
   <si>
     <t>CHARACTER / 스탯 분배</t>
+  </si>
+  <si>
+    <t>progression.status</t>
+  </si>
+  <si>
+    <t>progression</t>
+  </si>
+  <si>
+    <t>src/LevelProgress.tsx</t>
+  </si>
+  <si>
+    <t>레벨 {level} / {maxLevel} · 경험치 {exp} / {required}</t>
+  </si>
+  <si>
+    <t>{level}, {maxLevel}, {exp}, {required}</t>
+  </si>
+  <si>
+    <t>progression.maximum</t>
+  </si>
+  <si>
+    <t>레벨 {level} / {maxLevel} · 최고 레벨</t>
+  </si>
+  <si>
+    <t>{level}, {maxLevel}</t>
+  </si>
+  <si>
+    <t>progression.remaining</t>
+  </si>
+  <si>
+    <t>다음 레벨까지 경험치 {remaining}</t>
+  </si>
+  <si>
+    <t>{remaining}</t>
+  </si>
+  <si>
+    <t>progression.banked</t>
+  </si>
+  <si>
+    <t>보유 경험치 {exp}</t>
+  </si>
+  <si>
+    <t>{exp}</t>
+  </si>
+  <si>
+    <t>progression.label</t>
+  </si>
+  <si>
+    <t>레벨 경험치</t>
   </si>
 </sst>
 </file>
@@ -2973,7 +3021,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G306"/>
+  <dimension ref="A1:G311"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -10022,8 +10070,123 @@
         <v>22</v>
       </c>
     </row>
+    <row r="307" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A307" s="5" t="s">
+        <v>814</v>
+      </c>
+      <c r="B307" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="C307" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="D307" s="6" t="s">
+        <v>817</v>
+      </c>
+      <c r="E307" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F307" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G307" s="4" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="308" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A308" s="5" t="s">
+        <v>819</v>
+      </c>
+      <c r="B308" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="C308" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="D308" s="6" t="s">
+        <v>820</v>
+      </c>
+      <c r="E308" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F308" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G308" s="4" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="309" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A309" s="5" t="s">
+        <v>822</v>
+      </c>
+      <c r="B309" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="C309" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="D309" s="6" t="s">
+        <v>823</v>
+      </c>
+      <c r="E309" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F309" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G309" s="4" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="310" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A310" s="5" t="s">
+        <v>825</v>
+      </c>
+      <c r="B310" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="C310" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="D310" s="6" t="s">
+        <v>826</v>
+      </c>
+      <c r="E310" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F310" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G310" s="4" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="311" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A311" s="5" t="s">
+        <v>828</v>
+      </c>
+      <c r="B311" s="5" t="s">
+        <v>815</v>
+      </c>
+      <c r="C311" s="5" t="s">
+        <v>816</v>
+      </c>
+      <c r="D311" s="6" t="s">
+        <v>829</v>
+      </c>
+      <c r="E311" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F311" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G311" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G306"/>
+  <autoFilter ref="A1:G311"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Award and allocate two stat points per level
</commit_message>
<xml_diff>
--- a/content/game-texts.xlsx
+++ b/content/game-texts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2188" uniqueCount="830">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2251" uniqueCount="853">
   <si>
     <t>이매망량의 주인 — 산군 / 게임 텍스트 관리</t>
   </si>
@@ -2528,6 +2528,75 @@
   </si>
   <si>
     <t>레벨 경험치</t>
+  </si>
+  <si>
+    <t>growth.reward</t>
+  </si>
+  <si>
+    <t>growth</t>
+  </si>
+  <si>
+    <t>src/LevelUpAllocationPanel.tsx</t>
+  </si>
+  <si>
+    <t>스탯 포인트 {points} 획득</t>
+  </si>
+  <si>
+    <t>{points}</t>
+  </si>
+  <si>
+    <t>growth.open</t>
+  </si>
+  <si>
+    <t>레벨업 스탯 분배 ({points}P)</t>
+  </si>
+  <si>
+    <t>growth.title</t>
+  </si>
+  <si>
+    <t>레벨업 스탯 분배</t>
+  </si>
+  <si>
+    <t>growth.available</t>
+  </si>
+  <si>
+    <t>보유 포인트 {points} · 분배 예정 {spent} · 남길 포인트 {remaining}</t>
+  </si>
+  <si>
+    <t>{points}, {spent}, {remaining}</t>
+  </si>
+  <si>
+    <t>growth.help</t>
+  </si>
+  <si>
+    <t>레벨업마다 받은 포인트를 원하는 스탯에 분배하세요. 일부만 사용하고 나머지는 보관할 수 있습니다. 확정 후에는 되돌릴 수 없습니다.</t>
+  </si>
+  <si>
+    <t>growth.confirm</t>
+  </si>
+  <si>
+    <t>분배 확정</t>
+  </si>
+  <si>
+    <t>growth.back</t>
+  </si>
+  <si>
+    <t>게임으로 돌아가기</t>
+  </si>
+  <si>
+    <t>growth.preview</t>
+  </si>
+  <si>
+    <t>현재 {base} + 추가 {added} → {total}</t>
+  </si>
+  <si>
+    <t>{base}, {added}, {total}</t>
+  </si>
+  <si>
+    <t>growth.pending</t>
+  </si>
+  <si>
+    <t>미분배 스탯 포인트 {points}</t>
   </si>
 </sst>
 </file>
@@ -3021,7 +3090,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G311"/>
+  <dimension ref="A1:G320"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -10185,8 +10254,215 @@
         <v>22</v>
       </c>
     </row>
+    <row r="312" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A312" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="B312" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C312" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D312" s="6" t="s">
+        <v>833</v>
+      </c>
+      <c r="E312" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F312" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G312" s="4" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="313" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A313" s="5" t="s">
+        <v>835</v>
+      </c>
+      <c r="B313" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C313" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D313" s="6" t="s">
+        <v>836</v>
+      </c>
+      <c r="E313" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F313" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G313" s="4" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="314" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A314" s="5" t="s">
+        <v>837</v>
+      </c>
+      <c r="B314" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C314" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D314" s="6" t="s">
+        <v>838</v>
+      </c>
+      <c r="E314" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F314" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G314" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="315" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A315" s="5" t="s">
+        <v>839</v>
+      </c>
+      <c r="B315" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C315" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D315" s="6" t="s">
+        <v>840</v>
+      </c>
+      <c r="E315" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F315" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G315" s="4" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="316" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A316" s="5" t="s">
+        <v>842</v>
+      </c>
+      <c r="B316" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C316" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D316" s="6" t="s">
+        <v>843</v>
+      </c>
+      <c r="E316" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F316" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G316" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="317" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A317" s="5" t="s">
+        <v>844</v>
+      </c>
+      <c r="B317" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C317" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D317" s="6" t="s">
+        <v>845</v>
+      </c>
+      <c r="E317" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F317" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G317" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="318" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A318" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="B318" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C318" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D318" s="6" t="s">
+        <v>847</v>
+      </c>
+      <c r="E318" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F318" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G318" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="319" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A319" s="5" t="s">
+        <v>848</v>
+      </c>
+      <c r="B319" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C319" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D319" s="6" t="s">
+        <v>849</v>
+      </c>
+      <c r="E319" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F319" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G319" s="4" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="320" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A320" s="5" t="s">
+        <v>851</v>
+      </c>
+      <c r="B320" s="5" t="s">
+        <v>831</v>
+      </c>
+      <c r="C320" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="D320" s="6" t="s">
+        <v>852</v>
+      </c>
+      <c r="E320" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F320" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G320" s="4" t="s">
+        <v>834</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G311"/>
+  <autoFilter ref="A1:G320"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Split adventure events into battles, three-choice stories, and trading shops
</commit_message>
<xml_diff>
--- a/content/game-texts.xlsx
+++ b/content/game-texts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2251" uniqueCount="853">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2601" uniqueCount="961">
   <si>
     <t>이매망량의 주인 — 산군 / 게임 텍스트 관리</t>
   </si>
@@ -2597,6 +2597,330 @@
   </si>
   <si>
     <t>미분배 스탯 포인트 {points}</t>
+  </si>
+  <si>
+    <t>events.battle</t>
+  </si>
+  <si>
+    <t>events</t>
+  </si>
+  <si>
+    <t>src/game.ts / src/ShopPanel.tsx</t>
+  </si>
+  <si>
+    <t>전투</t>
+  </si>
+  <si>
+    <t>events.story</t>
+  </si>
+  <si>
+    <t>이야기</t>
+  </si>
+  <si>
+    <t>events.shop</t>
+  </si>
+  <si>
+    <t>상점</t>
+  </si>
+  <si>
+    <t>events.gate.trust</t>
+  </si>
+  <si>
+    <t>가면을 쓴 길잡이를 따라간다</t>
+  </si>
+  <si>
+    <t>events.gate.trust_hint</t>
+  </si>
+  <si>
+    <t>소지품을 잃고 저주에 걸립니다</t>
+  </si>
+  <si>
+    <t>events.gate.trust_result</t>
+  </si>
+  <si>
+    <t>길잡이는 안개 속으로 사라졌다. 행낭이 가벼워지고 싸늘한 기운이 몸에 남았다.</t>
+  </si>
+  <si>
+    <t>events.pool.offer</t>
+  </si>
+  <si>
+    <t>샘에 작은 공물을 바친다</t>
+  </si>
+  <si>
+    <t>events.pool.offer_hint</t>
+  </si>
+  <si>
+    <t>2냥 · 부적 획득</t>
+  </si>
+  <si>
+    <t>events.pool.offer_result</t>
+  </si>
+  <si>
+    <t>샘물이 잔잔해지며 삼재 부적을 밀어 올렸다.</t>
+  </si>
+  <si>
+    <t>events.camp.stranger</t>
+  </si>
+  <si>
+    <t>낯선 여행자에게 배낭을 맡긴다</t>
+  </si>
+  <si>
+    <t>events.camp.stranger_hint</t>
+  </si>
+  <si>
+    <t>아이템 손실 · 저주</t>
+  </si>
+  <si>
+    <t>events.camp.stranger_result</t>
+  </si>
+  <si>
+    <t>눈을 돌린 사이 여행자가 소지품을 가지고 달아났다. 모닥불이 푸르게 변했다.</t>
+  </si>
+  <si>
+    <t>events.bells.touch</t>
+  </si>
+  <si>
+    <t>붉은 글씨가 적힌 종을 만진다</t>
+  </si>
+  <si>
+    <t>events.bells.touch_hint</t>
+  </si>
+  <si>
+    <t>events.bells.touch_result</t>
+  </si>
+  <si>
+    <t>종에 묶인 원한이 손끝으로 스며들고 소지품 하나가 재로 변했다.</t>
+  </si>
+  <si>
+    <t>events.ambush.title</t>
+  </si>
+  <si>
+    <t>고갯길의 도깨비</t>
+  </si>
+  <si>
+    <t>events.ambush.place</t>
+  </si>
+  <si>
+    <t>한양 외곽 고개</t>
+  </si>
+  <si>
+    <t>events.ambush.text</t>
+  </si>
+  <si>
+    <t>몽둥이를 든 도깨비가 길 한가운데서 이를 드러낸다.</t>
+  </si>
+  <si>
+    <t>events.boss.title</t>
+  </si>
+  <si>
+    <t>대감신의 습격</t>
+  </si>
+  <si>
+    <t>events.boss.place</t>
+  </si>
+  <si>
+    <t>이름들의 나무 앞</t>
+  </si>
+  <si>
+    <t>events.boss.text</t>
+  </si>
+  <si>
+    <t>마지막 문 앞에 대감신이 나타났다. 잃어버린 이름을 되찾으려면 이 요괴를 쓰러뜨려야 한다.</t>
+  </si>
+  <si>
+    <t>events.blessing</t>
+  </si>
+  <si>
+    <t>산신의 가호</t>
+  </si>
+  <si>
+    <t>events.blessing.description</t>
+  </si>
+  <si>
+    <t>물리·주술 공격력과 방어력 +2</t>
+  </si>
+  <si>
+    <t>events.curse</t>
+  </si>
+  <si>
+    <t>원한의 저주</t>
+  </si>
+  <si>
+    <t>events.curse.description</t>
+  </si>
+  <si>
+    <t>물리·주술 공격력과 방어력 -2</t>
+  </si>
+  <si>
+    <t>events.effect.gain</t>
+  </si>
+  <si>
+    <t>{name} 획득 · {battles}회 전투 동안 적용</t>
+  </si>
+  <si>
+    <t>{name}, {battles}</t>
+  </si>
+  <si>
+    <t>events.effect.active</t>
+  </si>
+  <si>
+    <t>{name} · 남은 전투 {battles}회</t>
+  </si>
+  <si>
+    <t>events.item.gain</t>
+  </si>
+  <si>
+    <t>아이템 획득 · {name}</t>
+  </si>
+  <si>
+    <t>events.item.loss</t>
+  </si>
+  <si>
+    <t>아이템 손실 · {name}</t>
+  </si>
+  <si>
+    <t>events.item.none</t>
+  </si>
+  <si>
+    <t>잃을 아이템이 없어 3냥까지 잃었습니다.</t>
+  </si>
+  <si>
+    <t>events.drop.none</t>
+  </si>
+  <si>
+    <t>이번 전투에서는 아이템을 얻지 못했습니다.</t>
+  </si>
+  <si>
+    <t>items.potion.name</t>
+  </si>
+  <si>
+    <t>산삼 탕약</t>
+  </si>
+  <si>
+    <t>items.potion.description</t>
+  </si>
+  <si>
+    <t>자동 전투 중 체력 12 회복</t>
+  </si>
+  <si>
+    <t>shop.heading</t>
+  </si>
+  <si>
+    <t>구매와 판매</t>
+  </si>
+  <si>
+    <t>shop.gold</t>
+  </si>
+  <si>
+    <t>보유 금액 {gold}냥</t>
+  </si>
+  <si>
+    <t>{gold}</t>
+  </si>
+  <si>
+    <t>shop.row</t>
+  </si>
+  <si>
+    <t>구매 {buy}냥 · 판매 {sell}냥 · 보유 {count}개</t>
+  </si>
+  <si>
+    <t>{buy}, {sell}, {count}</t>
+  </si>
+  <si>
+    <t>shop.buy</t>
+  </si>
+  <si>
+    <t>{name} 구매</t>
+  </si>
+  <si>
+    <t>shop.sell</t>
+  </si>
+  <si>
+    <t>{name} 판매</t>
+  </si>
+  <si>
+    <t>shop.bought</t>
+  </si>
+  <si>
+    <t>{name} 구매 · {price}냥 지불</t>
+  </si>
+  <si>
+    <t>{name}, {price}</t>
+  </si>
+  <si>
+    <t>shop.sold</t>
+  </si>
+  <si>
+    <t>{name} 판매 · {price}냥 획득</t>
+  </si>
+  <si>
+    <t>shop.leave</t>
+  </si>
+  <si>
+    <t>상점을 나와 다음 길로</t>
+  </si>
+  <si>
+    <t>shop.journal</t>
+  </si>
+  <si>
+    <t>상점을 떠나 다음 길로 향했다.</t>
+  </si>
+  <si>
+    <t>shop.owned</t>
+  </si>
+  <si>
+    <t>이미 보유 중</t>
+  </si>
+  <si>
+    <t>shop.no_gold</t>
+  </si>
+  <si>
+    <t>금액 부족</t>
+  </si>
+  <si>
+    <t>shop.no_item</t>
+  </si>
+  <si>
+    <t>판매할 아이템 없음</t>
+  </si>
+  <si>
+    <t>events.drop.rate</t>
+  </si>
+  <si>
+    <t>아이템 획득 확률: 일반 40% · 보스 60%</t>
+  </si>
+  <si>
+    <t>events.types.help</t>
+  </si>
+  <si>
+    <t>전투에서 경험치를, 이야기에서 선택의 결과를, 상점에서 거래를 경험합니다.</t>
+  </si>
+  <si>
+    <t>events.item.duplicate</t>
+  </si>
+  <si>
+    <t>src/game.ts</t>
+  </si>
+  <si>
+    <t>이미 보유한 {name} 대신 {gold}냥을 받았습니다.</t>
+  </si>
+  <si>
+    <t>{name}, {gold}</t>
+  </si>
+  <si>
+    <t>events.transaction_log</t>
+  </si>
+  <si>
+    <t>{day}일 · {message}</t>
+  </si>
+  <si>
+    <t>{day}, {message}</t>
+  </si>
+  <si>
+    <t>shop.closed</t>
+  </si>
+  <si>
+    <t>지금은 거래할 수 없습니다.</t>
   </si>
 </sst>
 </file>
@@ -3090,7 +3414,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G320"/>
+  <dimension ref="A1:G370"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -10461,8 +10785,1158 @@
         <v>834</v>
       </c>
     </row>
+    <row r="321" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A321" s="5" t="s">
+        <v>853</v>
+      </c>
+      <c r="B321" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C321" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D321" s="6" t="s">
+        <v>856</v>
+      </c>
+      <c r="E321" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F321" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G321" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="322" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A322" s="5" t="s">
+        <v>857</v>
+      </c>
+      <c r="B322" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C322" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D322" s="6" t="s">
+        <v>858</v>
+      </c>
+      <c r="E322" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F322" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G322" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="323" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A323" s="5" t="s">
+        <v>859</v>
+      </c>
+      <c r="B323" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C323" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D323" s="6" t="s">
+        <v>860</v>
+      </c>
+      <c r="E323" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F323" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G323" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="324" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A324" s="5" t="s">
+        <v>861</v>
+      </c>
+      <c r="B324" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C324" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D324" s="6" t="s">
+        <v>862</v>
+      </c>
+      <c r="E324" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F324" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G324" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="325" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A325" s="5" t="s">
+        <v>863</v>
+      </c>
+      <c r="B325" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C325" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D325" s="6" t="s">
+        <v>864</v>
+      </c>
+      <c r="E325" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F325" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G325" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="326" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A326" s="5" t="s">
+        <v>865</v>
+      </c>
+      <c r="B326" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C326" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D326" s="6" t="s">
+        <v>866</v>
+      </c>
+      <c r="E326" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F326" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G326" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="327" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A327" s="5" t="s">
+        <v>867</v>
+      </c>
+      <c r="B327" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C327" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D327" s="6" t="s">
+        <v>868</v>
+      </c>
+      <c r="E327" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F327" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G327" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="328" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A328" s="5" t="s">
+        <v>869</v>
+      </c>
+      <c r="B328" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C328" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D328" s="6" t="s">
+        <v>870</v>
+      </c>
+      <c r="E328" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F328" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G328" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="329" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A329" s="5" t="s">
+        <v>871</v>
+      </c>
+      <c r="B329" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C329" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D329" s="6" t="s">
+        <v>872</v>
+      </c>
+      <c r="E329" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F329" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G329" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="330" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A330" s="5" t="s">
+        <v>873</v>
+      </c>
+      <c r="B330" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C330" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D330" s="6" t="s">
+        <v>874</v>
+      </c>
+      <c r="E330" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F330" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G330" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="331" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A331" s="5" t="s">
+        <v>875</v>
+      </c>
+      <c r="B331" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C331" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D331" s="6" t="s">
+        <v>876</v>
+      </c>
+      <c r="E331" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F331" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G331" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="332" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A332" s="5" t="s">
+        <v>877</v>
+      </c>
+      <c r="B332" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C332" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D332" s="6" t="s">
+        <v>878</v>
+      </c>
+      <c r="E332" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F332" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G332" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="333" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A333" s="5" t="s">
+        <v>879</v>
+      </c>
+      <c r="B333" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C333" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D333" s="6" t="s">
+        <v>880</v>
+      </c>
+      <c r="E333" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F333" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G333" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="334" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A334" s="5" t="s">
+        <v>881</v>
+      </c>
+      <c r="B334" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C334" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D334" s="6" t="s">
+        <v>876</v>
+      </c>
+      <c r="E334" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F334" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G334" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="335" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A335" s="5" t="s">
+        <v>882</v>
+      </c>
+      <c r="B335" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C335" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D335" s="6" t="s">
+        <v>883</v>
+      </c>
+      <c r="E335" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F335" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G335" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="336" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A336" s="5" t="s">
+        <v>884</v>
+      </c>
+      <c r="B336" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C336" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D336" s="6" t="s">
+        <v>885</v>
+      </c>
+      <c r="E336" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F336" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G336" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="337" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A337" s="5" t="s">
+        <v>886</v>
+      </c>
+      <c r="B337" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C337" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D337" s="6" t="s">
+        <v>887</v>
+      </c>
+      <c r="E337" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F337" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G337" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="338" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A338" s="5" t="s">
+        <v>888</v>
+      </c>
+      <c r="B338" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C338" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D338" s="6" t="s">
+        <v>889</v>
+      </c>
+      <c r="E338" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F338" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G338" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="339" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A339" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="B339" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C339" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D339" s="6" t="s">
+        <v>891</v>
+      </c>
+      <c r="E339" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F339" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G339" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="340" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A340" s="5" t="s">
+        <v>892</v>
+      </c>
+      <c r="B340" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C340" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D340" s="6" t="s">
+        <v>893</v>
+      </c>
+      <c r="E340" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F340" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G340" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="341" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A341" s="5" t="s">
+        <v>894</v>
+      </c>
+      <c r="B341" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C341" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D341" s="6" t="s">
+        <v>895</v>
+      </c>
+      <c r="E341" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F341" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G341" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="342" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A342" s="5" t="s">
+        <v>896</v>
+      </c>
+      <c r="B342" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C342" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D342" s="6" t="s">
+        <v>897</v>
+      </c>
+      <c r="E342" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F342" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G342" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="343" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A343" s="5" t="s">
+        <v>898</v>
+      </c>
+      <c r="B343" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C343" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D343" s="6" t="s">
+        <v>899</v>
+      </c>
+      <c r="E343" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F343" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G343" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="344" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A344" s="5" t="s">
+        <v>900</v>
+      </c>
+      <c r="B344" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C344" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D344" s="6" t="s">
+        <v>901</v>
+      </c>
+      <c r="E344" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F344" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G344" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="345" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A345" s="5" t="s">
+        <v>902</v>
+      </c>
+      <c r="B345" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C345" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D345" s="6" t="s">
+        <v>903</v>
+      </c>
+      <c r="E345" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F345" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G345" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="346" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A346" s="5" t="s">
+        <v>904</v>
+      </c>
+      <c r="B346" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C346" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D346" s="6" t="s">
+        <v>905</v>
+      </c>
+      <c r="E346" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F346" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G346" s="4" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="347" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A347" s="5" t="s">
+        <v>907</v>
+      </c>
+      <c r="B347" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C347" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D347" s="6" t="s">
+        <v>908</v>
+      </c>
+      <c r="E347" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F347" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G347" s="4" t="s">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="348" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A348" s="5" t="s">
+        <v>909</v>
+      </c>
+      <c r="B348" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C348" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D348" s="6" t="s">
+        <v>910</v>
+      </c>
+      <c r="E348" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F348" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G348" s="4" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="349" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A349" s="5" t="s">
+        <v>911</v>
+      </c>
+      <c r="B349" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C349" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D349" s="6" t="s">
+        <v>912</v>
+      </c>
+      <c r="E349" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F349" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G349" s="4" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="350" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A350" s="5" t="s">
+        <v>913</v>
+      </c>
+      <c r="B350" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C350" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D350" s="6" t="s">
+        <v>914</v>
+      </c>
+      <c r="E350" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F350" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G350" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="351" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A351" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="B351" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C351" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D351" s="6" t="s">
+        <v>916</v>
+      </c>
+      <c r="E351" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F351" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G351" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="352" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A352" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="B352" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C352" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D352" s="6" t="s">
+        <v>918</v>
+      </c>
+      <c r="E352" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F352" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G352" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="353" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A353" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="B353" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C353" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D353" s="6" t="s">
+        <v>920</v>
+      </c>
+      <c r="E353" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F353" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G353" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="354" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A354" s="5" t="s">
+        <v>921</v>
+      </c>
+      <c r="B354" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C354" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D354" s="6" t="s">
+        <v>922</v>
+      </c>
+      <c r="E354" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F354" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G354" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="355" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A355" s="5" t="s">
+        <v>923</v>
+      </c>
+      <c r="B355" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C355" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D355" s="6" t="s">
+        <v>924</v>
+      </c>
+      <c r="E355" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F355" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G355" s="4" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="356" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A356" s="5" t="s">
+        <v>926</v>
+      </c>
+      <c r="B356" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C356" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D356" s="6" t="s">
+        <v>927</v>
+      </c>
+      <c r="E356" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F356" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G356" s="4" t="s">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="357" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A357" s="5" t="s">
+        <v>929</v>
+      </c>
+      <c r="B357" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C357" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D357" s="6" t="s">
+        <v>930</v>
+      </c>
+      <c r="E357" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F357" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G357" s="4" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="358" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A358" s="5" t="s">
+        <v>931</v>
+      </c>
+      <c r="B358" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C358" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D358" s="6" t="s">
+        <v>932</v>
+      </c>
+      <c r="E358" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F358" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G358" s="4" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="359" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A359" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="B359" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C359" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D359" s="6" t="s">
+        <v>934</v>
+      </c>
+      <c r="E359" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F359" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G359" s="4" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="360" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A360" s="5" t="s">
+        <v>936</v>
+      </c>
+      <c r="B360" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C360" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D360" s="6" t="s">
+        <v>937</v>
+      </c>
+      <c r="E360" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F360" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G360" s="4" t="s">
+        <v>935</v>
+      </c>
+    </row>
+    <row r="361" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A361" s="5" t="s">
+        <v>938</v>
+      </c>
+      <c r="B361" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C361" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D361" s="6" t="s">
+        <v>939</v>
+      </c>
+      <c r="E361" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F361" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G361" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="362" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A362" s="5" t="s">
+        <v>940</v>
+      </c>
+      <c r="B362" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C362" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D362" s="6" t="s">
+        <v>941</v>
+      </c>
+      <c r="E362" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F362" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G362" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="363" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A363" s="5" t="s">
+        <v>942</v>
+      </c>
+      <c r="B363" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C363" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D363" s="6" t="s">
+        <v>943</v>
+      </c>
+      <c r="E363" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F363" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G363" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="364" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A364" s="5" t="s">
+        <v>944</v>
+      </c>
+      <c r="B364" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C364" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D364" s="6" t="s">
+        <v>945</v>
+      </c>
+      <c r="E364" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F364" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G364" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="365" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A365" s="5" t="s">
+        <v>946</v>
+      </c>
+      <c r="B365" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C365" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D365" s="6" t="s">
+        <v>947</v>
+      </c>
+      <c r="E365" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F365" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G365" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="366" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A366" s="5" t="s">
+        <v>948</v>
+      </c>
+      <c r="B366" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C366" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D366" s="6" t="s">
+        <v>949</v>
+      </c>
+      <c r="E366" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F366" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G366" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="367" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A367" s="5" t="s">
+        <v>950</v>
+      </c>
+      <c r="B367" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C367" s="5" t="s">
+        <v>855</v>
+      </c>
+      <c r="D367" s="6" t="s">
+        <v>951</v>
+      </c>
+      <c r="E367" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F367" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G367" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="368" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A368" s="5" t="s">
+        <v>952</v>
+      </c>
+      <c r="B368" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C368" s="5" t="s">
+        <v>953</v>
+      </c>
+      <c r="D368" s="6" t="s">
+        <v>954</v>
+      </c>
+      <c r="E368" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F368" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G368" s="4" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="369" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A369" s="5" t="s">
+        <v>956</v>
+      </c>
+      <c r="B369" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C369" s="5" t="s">
+        <v>953</v>
+      </c>
+      <c r="D369" s="6" t="s">
+        <v>957</v>
+      </c>
+      <c r="E369" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F369" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G369" s="4" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="370" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A370" s="5" t="s">
+        <v>959</v>
+      </c>
+      <c r="B370" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="C370" s="5" t="s">
+        <v>953</v>
+      </c>
+      <c r="D370" s="6" t="s">
+        <v>960</v>
+      </c>
+      <c r="E370" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F370" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G370" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G320"/>
+  <autoFilter ref="A1:G370"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Manage monster encounters and drop tables in Excel
</commit_message>
<xml_diff>
--- a/content/game-texts.xlsx
+++ b/content/game-texts.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2776" uniqueCount="1020">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2748" uniqueCount="1011">
   <si>
     <t>이매망량의 주인 — 산군 / 게임 텍스트 관리</t>
   </si>
@@ -1729,33 +1729,6 @@
     <t>{day}, {title}, {label}, {result}</t>
   </si>
   <si>
-    <t>game.157</t>
-  </si>
-  <si>
-    <t>src/game.ts:187</t>
-  </si>
-  <si>
-    <t>이름을 삼키는 대감신</t>
-  </si>
-  <si>
-    <t>game.158</t>
-  </si>
-  <si>
-    <t>창에 묶인 묵은 삵</t>
-  </si>
-  <si>
-    <t>game.159</t>
-  </si>
-  <si>
-    <t>목소리를 훔친 원귀</t>
-  </si>
-  <si>
-    <t>game.160</t>
-  </si>
-  <si>
-    <t>성문 밖 도깨비</t>
-  </si>
-  <si>
     <t>game.161</t>
   </si>
   <si>
@@ -2827,7 +2800,7 @@
     <t>events.drop.rate</t>
   </si>
   <si>
-    <t>아이템 획득 확률: 일반 40% · 보스 60%</t>
+    <t>드랍 확률과 등장 몬스터는 몬스터별 설정을 따릅니다. 이미 가진 장비는 중복 지급되지 않습니다.</t>
   </si>
   <si>
     <t>events.types.help</t>
@@ -3591,7 +3564,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G395"/>
+  <dimension ref="A1:G391"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -8774,21 +8747,21 @@
         <v>22</v>
       </c>
       <c r="G225" s="4" t="s">
-        <v>22</v>
+        <v>567</v>
       </c>
     </row>
     <row r="226" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A226" s="5" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B226" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C226" s="5" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="D226" s="6" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="E226" s="7" t="s">
         <v>22</v>
@@ -8802,16 +8775,16 @@
     </row>
     <row r="227" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A227" s="5" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="B227" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C227" s="5" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
       <c r="D227" s="6" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="E227" s="7" t="s">
         <v>22</v>
@@ -8825,16 +8798,16 @@
     </row>
     <row r="228" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A228" s="5" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B228" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C228" s="5" t="s">
-        <v>565</v>
+        <v>575</v>
       </c>
       <c r="D228" s="6" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="E228" s="7" t="s">
         <v>22</v>
@@ -8848,16 +8821,16 @@
     </row>
     <row r="229" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A229" s="5" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="B229" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C229" s="5" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="D229" s="6" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="E229" s="7" t="s">
         <v>22</v>
@@ -8866,21 +8839,21 @@
         <v>22</v>
       </c>
       <c r="G229" s="4" t="s">
-        <v>576</v>
+        <v>22</v>
       </c>
     </row>
     <row r="230" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A230" s="5" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B230" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C230" s="5" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D230" s="6" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E230" s="7" t="s">
         <v>22</v>
@@ -8894,16 +8867,16 @@
     </row>
     <row r="231" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="5" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="B231" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C231" s="5" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="D231" s="6" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E231" s="7" t="s">
         <v>22</v>
@@ -8912,21 +8885,21 @@
         <v>22</v>
       </c>
       <c r="G231" s="4" t="s">
-        <v>22</v>
+        <v>586</v>
       </c>
     </row>
     <row r="232" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A232" s="5" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="B232" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C232" s="5" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="D232" s="6" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="E232" s="7" t="s">
         <v>22</v>
@@ -8940,16 +8913,16 @@
     </row>
     <row r="233" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A233" s="5" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="B233" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C233" s="5" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D233" s="6" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E233" s="7" t="s">
         <v>22</v>
@@ -8958,21 +8931,21 @@
         <v>22</v>
       </c>
       <c r="G233" s="4" t="s">
-        <v>22</v>
+        <v>592</v>
       </c>
     </row>
     <row r="234" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A234" s="5" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="B234" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C234" s="5" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="D234" s="6" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="E234" s="7" t="s">
         <v>22</v>
@@ -8986,16 +8959,16 @@
     </row>
     <row r="235" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A235" s="5" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="B235" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C235" s="5" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="D235" s="6" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="E235" s="7" t="s">
         <v>22</v>
@@ -9004,21 +8977,21 @@
         <v>22</v>
       </c>
       <c r="G235" s="4" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
     </row>
     <row r="236" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A236" s="5" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="B236" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C236" s="5" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="D236" s="6" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="E236" s="7" t="s">
         <v>22</v>
@@ -9032,16 +9005,16 @@
     </row>
     <row r="237" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A237" s="5" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="B237" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C237" s="5" t="s">
-        <v>597</v>
+        <v>604</v>
       </c>
       <c r="D237" s="6" t="s">
-        <v>600</v>
+        <v>605</v>
       </c>
       <c r="E237" s="7" t="s">
         <v>22</v>
@@ -9050,21 +9023,21 @@
         <v>22</v>
       </c>
       <c r="G237" s="4" t="s">
-        <v>601</v>
+        <v>22</v>
       </c>
     </row>
     <row r="238" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A238" s="5" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="B238" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C238" s="5" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="D238" s="6" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="E238" s="7" t="s">
         <v>22</v>
@@ -9078,16 +9051,16 @@
     </row>
     <row r="239" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A239" s="5" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B239" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C239" s="5" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="D239" s="6" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E239" s="7" t="s">
         <v>22</v>
@@ -9096,18 +9069,18 @@
         <v>22</v>
       </c>
       <c r="G239" s="4" t="s">
-        <v>608</v>
+        <v>22</v>
       </c>
     </row>
     <row r="240" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A240" s="5" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B240" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C240" s="5" t="s">
-        <v>610</v>
+        <v>604</v>
       </c>
       <c r="D240" s="6" t="s">
         <v>611</v>
@@ -9153,10 +9126,10 @@
         <v>212</v>
       </c>
       <c r="C242" s="5" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="D242" s="6" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="E242" s="7" t="s">
         <v>22</v>
@@ -9170,16 +9143,16 @@
     </row>
     <row r="243" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A243" s="5" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B243" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C243" s="5" t="s">
-        <v>613</v>
+        <v>619</v>
       </c>
       <c r="D243" s="6" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E243" s="7" t="s">
         <v>22</v>
@@ -9193,16 +9166,16 @@
     </row>
     <row r="244" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A244" s="5" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="B244" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C244" s="5" t="s">
-        <v>613</v>
+        <v>622</v>
       </c>
       <c r="D244" s="6" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="E244" s="7" t="s">
         <v>22</v>
@@ -9211,21 +9184,21 @@
         <v>22</v>
       </c>
       <c r="G244" s="4" t="s">
-        <v>22</v>
+        <v>624</v>
       </c>
     </row>
     <row r="245" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A245" s="5" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="B245" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C245" s="5" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="D245" s="6" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="E245" s="7" t="s">
         <v>22</v>
@@ -9239,16 +9212,16 @@
     </row>
     <row r="246" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A246" s="5" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="B246" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C246" s="5" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="D246" s="6" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="E246" s="7" t="s">
         <v>22</v>
@@ -9262,16 +9235,16 @@
     </row>
     <row r="247" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A247" s="5" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="B247" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C247" s="5" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="D247" s="6" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="E247" s="7" t="s">
         <v>22</v>
@@ -9280,21 +9253,21 @@
         <v>22</v>
       </c>
       <c r="G247" s="4" t="s">
-        <v>22</v>
+        <v>632</v>
       </c>
     </row>
     <row r="248" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A248" s="5" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B248" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C248" s="5" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D248" s="6" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="E248" s="7" t="s">
         <v>22</v>
@@ -9303,21 +9276,21 @@
         <v>22</v>
       </c>
       <c r="G248" s="4" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
     </row>
     <row r="249" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A249" s="5" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="B249" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C249" s="5" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="D249" s="6" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E249" s="7" t="s">
         <v>22</v>
@@ -9326,21 +9299,21 @@
         <v>22</v>
       </c>
       <c r="G249" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="250" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A250" s="5" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="B250" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C250" s="5" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="D250" s="6" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="E250" s="7" t="s">
         <v>22</v>
@@ -9349,21 +9322,21 @@
         <v>22</v>
       </c>
       <c r="G250" s="4" t="s">
-        <v>22</v>
+        <v>643</v>
       </c>
     </row>
     <row r="251" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A251" s="5" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="B251" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C251" s="5" t="s">
-        <v>635</v>
+        <v>645</v>
       </c>
       <c r="D251" s="6" t="s">
-        <v>640</v>
+        <v>646</v>
       </c>
       <c r="E251" s="7" t="s">
         <v>22</v>
@@ -9372,21 +9345,21 @@
         <v>22</v>
       </c>
       <c r="G251" s="4" t="s">
-        <v>641</v>
+        <v>647</v>
       </c>
     </row>
     <row r="252" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A252" s="5" t="s">
-        <v>642</v>
+        <v>648</v>
       </c>
       <c r="B252" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C252" s="5" t="s">
-        <v>643</v>
+        <v>649</v>
       </c>
       <c r="D252" s="6" t="s">
-        <v>644</v>
+        <v>650</v>
       </c>
       <c r="E252" s="7" t="s">
         <v>22</v>
@@ -9395,21 +9368,21 @@
         <v>22</v>
       </c>
       <c r="G252" s="4" t="s">
-        <v>645</v>
+        <v>651</v>
       </c>
     </row>
     <row r="253" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A253" s="5" t="s">
-        <v>646</v>
+        <v>652</v>
       </c>
       <c r="B253" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C253" s="5" t="s">
-        <v>647</v>
+        <v>653</v>
       </c>
       <c r="D253" s="6" t="s">
-        <v>648</v>
+        <v>654</v>
       </c>
       <c r="E253" s="7" t="s">
         <v>22</v>
@@ -9418,21 +9391,21 @@
         <v>22</v>
       </c>
       <c r="G253" s="4" t="s">
-        <v>649</v>
+        <v>567</v>
       </c>
     </row>
     <row r="254" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A254" s="5" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="B254" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C254" s="5" t="s">
-        <v>647</v>
+        <v>656</v>
       </c>
       <c r="D254" s="6" t="s">
-        <v>651</v>
+        <v>657</v>
       </c>
       <c r="E254" s="7" t="s">
         <v>22</v>
@@ -9441,21 +9414,21 @@
         <v>22</v>
       </c>
       <c r="G254" s="4" t="s">
-        <v>652</v>
+        <v>658</v>
       </c>
     </row>
     <row r="255" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A255" s="5" t="s">
-        <v>653</v>
+        <v>659</v>
       </c>
       <c r="B255" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C255" s="5" t="s">
-        <v>654</v>
+        <v>660</v>
       </c>
       <c r="D255" s="6" t="s">
-        <v>655</v>
+        <v>661</v>
       </c>
       <c r="E255" s="7" t="s">
         <v>22</v>
@@ -9464,21 +9437,21 @@
         <v>22</v>
       </c>
       <c r="G255" s="4" t="s">
-        <v>656</v>
+        <v>22</v>
       </c>
     </row>
     <row r="256" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A256" s="5" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="B256" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C256" s="5" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="D256" s="6" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="E256" s="7" t="s">
         <v>22</v>
@@ -9487,21 +9460,21 @@
         <v>22</v>
       </c>
       <c r="G256" s="4" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
     </row>
     <row r="257" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A257" s="5" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="B257" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C257" s="5" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="D257" s="6" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="E257" s="7" t="s">
         <v>22</v>
@@ -9510,21 +9483,21 @@
         <v>22</v>
       </c>
       <c r="G257" s="4" t="s">
-        <v>576</v>
+        <v>651</v>
       </c>
     </row>
     <row r="258" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A258" s="5" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B258" s="5" t="s">
         <v>212</v>
       </c>
       <c r="C258" s="5" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="D258" s="6" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="E258" s="7" t="s">
         <v>22</v>
@@ -9533,21 +9506,21 @@
         <v>22</v>
       </c>
       <c r="G258" s="4" t="s">
-        <v>667</v>
+        <v>22</v>
       </c>
     </row>
     <row r="259" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A259" s="5" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>212</v>
+        <v>672</v>
       </c>
       <c r="C259" s="5" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D259" s="6" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="E259" s="7" t="s">
         <v>22</v>
@@ -9561,16 +9534,16 @@
     </row>
     <row r="260" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A260" s="5" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>212</v>
+        <v>672</v>
       </c>
       <c r="C260" s="5" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D260" s="6" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="E260" s="7" t="s">
         <v>22</v>
@@ -9579,21 +9552,21 @@
         <v>22</v>
       </c>
       <c r="G260" s="4" t="s">
-        <v>673</v>
+        <v>22</v>
       </c>
     </row>
     <row r="261" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A261" s="5" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>212</v>
+        <v>672</v>
       </c>
       <c r="C261" s="5" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="D261" s="6" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="E261" s="7" t="s">
         <v>22</v>
@@ -9602,21 +9575,21 @@
         <v>22</v>
       </c>
       <c r="G261" s="4" t="s">
-        <v>660</v>
+        <v>22</v>
       </c>
     </row>
     <row r="262" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A262" s="5" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="B262" s="5" t="s">
-        <v>212</v>
+        <v>672</v>
       </c>
       <c r="C262" s="5" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="D262" s="6" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="E262" s="7" t="s">
         <v>22</v>
@@ -9625,21 +9598,21 @@
         <v>22</v>
       </c>
       <c r="G262" s="4" t="s">
-        <v>22</v>
+        <v>682</v>
       </c>
     </row>
     <row r="263" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A263" s="5" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="B263" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C263" s="5" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="D263" s="6" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="E263" s="7" t="s">
         <v>22</v>
@@ -9648,21 +9621,21 @@
         <v>22</v>
       </c>
       <c r="G263" s="4" t="s">
-        <v>22</v>
+        <v>686</v>
       </c>
     </row>
     <row r="264" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A264" s="5" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C264" s="5" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="D264" s="6" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="E264" s="7" t="s">
         <v>22</v>
@@ -9676,16 +9649,16 @@
     </row>
     <row r="265" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A265" s="5" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="B265" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C265" s="5" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="D265" s="6" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E265" s="7" t="s">
         <v>22</v>
@@ -9694,21 +9667,21 @@
         <v>22</v>
       </c>
       <c r="G265" s="4" t="s">
-        <v>22</v>
+        <v>692</v>
       </c>
     </row>
     <row r="266" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A266" s="5" t="s">
-        <v>688</v>
+        <v>693</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C266" s="5" t="s">
-        <v>689</v>
+        <v>694</v>
       </c>
       <c r="D266" s="6" t="s">
-        <v>690</v>
+        <v>695</v>
       </c>
       <c r="E266" s="7" t="s">
         <v>22</v>
@@ -9717,21 +9690,21 @@
         <v>22</v>
       </c>
       <c r="G266" s="4" t="s">
-        <v>691</v>
+        <v>640</v>
       </c>
     </row>
     <row r="267" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A267" s="5" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C267" s="5" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="D267" s="6" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="E267" s="7" t="s">
         <v>22</v>
@@ -9740,21 +9713,21 @@
         <v>22</v>
       </c>
       <c r="G267" s="4" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
     </row>
     <row r="268" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A268" s="5" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="B268" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C268" s="5" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="D268" s="6" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="E268" s="7" t="s">
         <v>22</v>
@@ -9768,16 +9741,16 @@
     </row>
     <row r="269" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A269" s="5" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="B269" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C269" s="5" t="s">
-        <v>697</v>
+        <v>704</v>
       </c>
       <c r="D269" s="6" t="s">
-        <v>700</v>
+        <v>705</v>
       </c>
       <c r="E269" s="7" t="s">
         <v>22</v>
@@ -9786,21 +9759,21 @@
         <v>22</v>
       </c>
       <c r="G269" s="4" t="s">
-        <v>701</v>
+        <v>22</v>
       </c>
     </row>
     <row r="270" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A270" s="5" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="B270" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C270" s="5" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="D270" s="6" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="E270" s="7" t="s">
         <v>22</v>
@@ -9809,21 +9782,21 @@
         <v>22</v>
       </c>
       <c r="G270" s="4" t="s">
-        <v>649</v>
+        <v>22</v>
       </c>
     </row>
     <row r="271" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A271" s="5" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="B271" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C271" s="5" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="D271" s="6" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="E271" s="7" t="s">
         <v>22</v>
@@ -9832,21 +9805,21 @@
         <v>22</v>
       </c>
       <c r="G271" s="4" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
     </row>
     <row r="272" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A272" s="5" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C272" s="5" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="D272" s="6" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="E272" s="7" t="s">
         <v>22</v>
@@ -9855,21 +9828,21 @@
         <v>22</v>
       </c>
       <c r="G272" s="4" t="s">
-        <v>22</v>
+        <v>716</v>
       </c>
     </row>
     <row r="273" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A273" s="5" t="s">
-        <v>712</v>
+        <v>717</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C273" s="5" t="s">
-        <v>713</v>
+        <v>718</v>
       </c>
       <c r="D273" s="6" t="s">
-        <v>714</v>
+        <v>719</v>
       </c>
       <c r="E273" s="7" t="s">
         <v>22</v>
@@ -9883,16 +9856,16 @@
     </row>
     <row r="274" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A274" s="5" t="s">
-        <v>715</v>
+        <v>720</v>
       </c>
       <c r="B274" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C274" s="5" t="s">
-        <v>716</v>
+        <v>721</v>
       </c>
       <c r="D274" s="6" t="s">
-        <v>717</v>
+        <v>722</v>
       </c>
       <c r="E274" s="7" t="s">
         <v>22</v>
@@ -9906,16 +9879,16 @@
     </row>
     <row r="275" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A275" s="5" t="s">
-        <v>718</v>
+        <v>723</v>
       </c>
       <c r="B275" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C275" s="5" t="s">
-        <v>719</v>
+        <v>724</v>
       </c>
       <c r="D275" s="6" t="s">
-        <v>720</v>
+        <v>725</v>
       </c>
       <c r="E275" s="7" t="s">
         <v>22</v>
@@ -9924,21 +9897,21 @@
         <v>22</v>
       </c>
       <c r="G275" s="4" t="s">
-        <v>721</v>
+        <v>726</v>
       </c>
     </row>
     <row r="276" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A276" s="5" t="s">
-        <v>722</v>
+        <v>727</v>
       </c>
       <c r="B276" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C276" s="5" t="s">
-        <v>723</v>
+        <v>728</v>
       </c>
       <c r="D276" s="6" t="s">
-        <v>724</v>
+        <v>729</v>
       </c>
       <c r="E276" s="7" t="s">
         <v>22</v>
@@ -9947,21 +9920,21 @@
         <v>22</v>
       </c>
       <c r="G276" s="4" t="s">
-        <v>725</v>
+        <v>730</v>
       </c>
     </row>
     <row r="277" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A277" s="5" t="s">
-        <v>726</v>
+        <v>731</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C277" s="5" t="s">
-        <v>727</v>
+        <v>732</v>
       </c>
       <c r="D277" s="6" t="s">
-        <v>728</v>
+        <v>733</v>
       </c>
       <c r="E277" s="7" t="s">
         <v>22</v>
@@ -9970,21 +9943,21 @@
         <v>22</v>
       </c>
       <c r="G277" s="4" t="s">
-        <v>22</v>
+        <v>734</v>
       </c>
     </row>
     <row r="278" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A278" s="5" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="B278" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C278" s="5" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="D278" s="6" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
       <c r="E278" s="7" t="s">
         <v>22</v>
@@ -9993,21 +9966,21 @@
         <v>22</v>
       </c>
       <c r="G278" s="4" t="s">
-        <v>22</v>
+        <v>510</v>
       </c>
     </row>
     <row r="279" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A279" s="5" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B279" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C279" s="5" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="D279" s="6" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="E279" s="7" t="s">
         <v>22</v>
@@ -10016,21 +9989,21 @@
         <v>22</v>
       </c>
       <c r="G279" s="4" t="s">
-        <v>735</v>
+        <v>180</v>
       </c>
     </row>
     <row r="280" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A280" s="5" t="s">
-        <v>736</v>
+        <v>741</v>
       </c>
       <c r="B280" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C280" s="5" t="s">
-        <v>737</v>
+        <v>742</v>
       </c>
       <c r="D280" s="6" t="s">
-        <v>738</v>
+        <v>743</v>
       </c>
       <c r="E280" s="7" t="s">
         <v>22</v>
@@ -10039,21 +10012,21 @@
         <v>22</v>
       </c>
       <c r="G280" s="4" t="s">
-        <v>739</v>
+        <v>22</v>
       </c>
     </row>
     <row r="281" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A281" s="5" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="B281" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C281" s="5" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="D281" s="6" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="E281" s="7" t="s">
         <v>22</v>
@@ -10062,21 +10035,21 @@
         <v>22</v>
       </c>
       <c r="G281" s="4" t="s">
-        <v>743</v>
+        <v>180</v>
       </c>
     </row>
     <row r="282" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A282" s="5" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="B282" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C282" s="5" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="D282" s="6" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="E282" s="7" t="s">
         <v>22</v>
@@ -10085,21 +10058,21 @@
         <v>22</v>
       </c>
       <c r="G282" s="4" t="s">
-        <v>510</v>
+        <v>22</v>
       </c>
     </row>
     <row r="283" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A283" s="5" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="B283" s="5" t="s">
-        <v>681</v>
+        <v>672</v>
       </c>
       <c r="C283" s="5" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="D283" s="6" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="E283" s="7" t="s">
         <v>22</v>
@@ -10108,21 +10081,21 @@
         <v>22</v>
       </c>
       <c r="G283" s="4" t="s">
-        <v>180</v>
+        <v>22</v>
       </c>
     </row>
     <row r="284" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A284" s="5" t="s">
+        <v>752</v>
+      </c>
+      <c r="B284" s="5" t="s">
+        <v>672</v>
+      </c>
+      <c r="C284" s="5" t="s">
         <v>750</v>
       </c>
-      <c r="B284" s="5" t="s">
-        <v>681</v>
-      </c>
-      <c r="C284" s="5" t="s">
-        <v>751</v>
-      </c>
       <c r="D284" s="6" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="E284" s="7" t="s">
         <v>22</v>
@@ -10136,16 +10109,16 @@
     </row>
     <row r="285" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A285" s="5" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="B285" s="5" t="s">
-        <v>681</v>
+        <v>755</v>
       </c>
       <c r="C285" s="5" t="s">
-        <v>751</v>
+        <v>756</v>
       </c>
       <c r="D285" s="6" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="E285" s="7" t="s">
         <v>22</v>
@@ -10154,21 +10127,21 @@
         <v>22</v>
       </c>
       <c r="G285" s="4" t="s">
-        <v>180</v>
+        <v>22</v>
       </c>
     </row>
     <row r="286" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A286" s="5" t="s">
+        <v>758</v>
+      </c>
+      <c r="B286" s="5" t="s">
         <v>755</v>
       </c>
-      <c r="B286" s="5" t="s">
-        <v>681</v>
-      </c>
       <c r="C286" s="5" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="D286" s="6" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="E286" s="7" t="s">
         <v>22</v>
@@ -10177,21 +10150,21 @@
         <v>22</v>
       </c>
       <c r="G286" s="4" t="s">
-        <v>22</v>
+        <v>761</v>
       </c>
     </row>
     <row r="287" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A287" s="5" t="s">
-        <v>758</v>
+        <v>762</v>
       </c>
       <c r="B287" s="5" t="s">
-        <v>681</v>
+        <v>755</v>
       </c>
       <c r="C287" s="5" t="s">
-        <v>759</v>
+        <v>763</v>
       </c>
       <c r="D287" s="6" t="s">
-        <v>760</v>
+        <v>764</v>
       </c>
       <c r="E287" s="7" t="s">
         <v>22</v>
@@ -10205,16 +10178,16 @@
     </row>
     <row r="288" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A288" s="5" t="s">
-        <v>761</v>
+        <v>765</v>
       </c>
       <c r="B288" s="5" t="s">
-        <v>681</v>
+        <v>755</v>
       </c>
       <c r="C288" s="5" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
       <c r="D288" s="6" t="s">
-        <v>762</v>
+        <v>767</v>
       </c>
       <c r="E288" s="7" t="s">
         <v>22</v>
@@ -10223,21 +10196,21 @@
         <v>22</v>
       </c>
       <c r="G288" s="4" t="s">
-        <v>22</v>
+        <v>510</v>
       </c>
     </row>
     <row r="289" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A289" s="5" t="s">
-        <v>763</v>
+        <v>768</v>
       </c>
       <c r="B289" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C289" s="5" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="D289" s="6" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
       <c r="E289" s="7" t="s">
         <v>22</v>
@@ -10246,21 +10219,21 @@
         <v>22</v>
       </c>
       <c r="G289" s="4" t="s">
-        <v>22</v>
+        <v>510</v>
       </c>
     </row>
     <row r="290" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A290" s="5" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
       <c r="B290" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C290" s="5" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="D290" s="6" t="s">
-        <v>769</v>
+        <v>772</v>
       </c>
       <c r="E290" s="7" t="s">
         <v>22</v>
@@ -10269,21 +10242,21 @@
         <v>22</v>
       </c>
       <c r="G290" s="4" t="s">
-        <v>770</v>
+        <v>180</v>
       </c>
     </row>
     <row r="291" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A291" s="5" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="B291" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C291" s="5" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="D291" s="6" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="E291" s="7" t="s">
         <v>22</v>
@@ -10292,21 +10265,21 @@
         <v>22</v>
       </c>
       <c r="G291" s="4" t="s">
-        <v>22</v>
+        <v>180</v>
       </c>
     </row>
     <row r="292" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A292" s="5" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="B292" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C292" s="5" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="D292" s="6" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="E292" s="7" t="s">
         <v>22</v>
@@ -10315,21 +10288,21 @@
         <v>22</v>
       </c>
       <c r="G292" s="4" t="s">
-        <v>510</v>
+        <v>22</v>
       </c>
     </row>
     <row r="293" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A293" s="5" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="B293" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C293" s="5" t="s">
-        <v>775</v>
+        <v>780</v>
       </c>
       <c r="D293" s="6" t="s">
-        <v>778</v>
+        <v>781</v>
       </c>
       <c r="E293" s="7" t="s">
         <v>22</v>
@@ -10338,21 +10311,21 @@
         <v>22</v>
       </c>
       <c r="G293" s="4" t="s">
-        <v>510</v>
+        <v>22</v>
       </c>
     </row>
     <row r="294" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A294" s="5" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
       <c r="B294" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C294" s="5" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="D294" s="6" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="E294" s="7" t="s">
         <v>22</v>
@@ -10361,21 +10334,21 @@
         <v>22</v>
       </c>
       <c r="G294" s="4" t="s">
-        <v>180</v>
+        <v>22</v>
       </c>
     </row>
     <row r="295" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A295" s="5" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="B295" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C295" s="5" t="s">
         <v>783</v>
       </c>
       <c r="D295" s="6" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="E295" s="7" t="s">
         <v>22</v>
@@ -10384,21 +10357,21 @@
         <v>22</v>
       </c>
       <c r="G295" s="4" t="s">
-        <v>180</v>
+        <v>22</v>
       </c>
     </row>
     <row r="296" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A296" s="5" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="B296" s="5" t="s">
-        <v>764</v>
+        <v>755</v>
       </c>
       <c r="C296" s="5" t="s">
-        <v>786</v>
+        <v>783</v>
       </c>
       <c r="D296" s="6" t="s">
-        <v>787</v>
+        <v>788</v>
       </c>
       <c r="E296" s="7" t="s">
         <v>22</v>
@@ -10412,16 +10385,16 @@
     </row>
     <row r="297" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A297" s="5" t="s">
-        <v>788</v>
+        <v>789</v>
       </c>
       <c r="B297" s="5" t="s">
-        <v>764</v>
+        <v>790</v>
       </c>
       <c r="C297" s="5" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="D297" s="6" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="E297" s="7" t="s">
         <v>22</v>
@@ -10430,21 +10403,21 @@
         <v>22</v>
       </c>
       <c r="G297" s="4" t="s">
-        <v>22</v>
+        <v>793</v>
       </c>
     </row>
     <row r="298" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A298" s="5" t="s">
+        <v>794</v>
+      </c>
+      <c r="B298" s="5" t="s">
+        <v>790</v>
+      </c>
+      <c r="C298" s="5" t="s">
         <v>791</v>
       </c>
-      <c r="B298" s="5" t="s">
-        <v>764</v>
-      </c>
-      <c r="C298" s="5" t="s">
-        <v>792</v>
-      </c>
       <c r="D298" s="6" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="E298" s="7" t="s">
         <v>22</v>
@@ -10453,21 +10426,21 @@
         <v>22</v>
       </c>
       <c r="G298" s="4" t="s">
-        <v>22</v>
+        <v>796</v>
       </c>
     </row>
     <row r="299" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A299" s="5" t="s">
-        <v>794</v>
+        <v>797</v>
       </c>
       <c r="B299" s="5" t="s">
-        <v>764</v>
+        <v>790</v>
       </c>
       <c r="C299" s="5" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="D299" s="6" t="s">
-        <v>795</v>
+        <v>798</v>
       </c>
       <c r="E299" s="7" t="s">
         <v>22</v>
@@ -10476,21 +10449,21 @@
         <v>22</v>
       </c>
       <c r="G299" s="4" t="s">
-        <v>22</v>
+        <v>799</v>
       </c>
     </row>
     <row r="300" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A300" s="5" t="s">
-        <v>796</v>
+        <v>800</v>
       </c>
       <c r="B300" s="5" t="s">
-        <v>764</v>
+        <v>790</v>
       </c>
       <c r="C300" s="5" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="D300" s="6" t="s">
-        <v>797</v>
+        <v>801</v>
       </c>
       <c r="E300" s="7" t="s">
         <v>22</v>
@@ -10499,21 +10472,21 @@
         <v>22</v>
       </c>
       <c r="G300" s="4" t="s">
-        <v>22</v>
+        <v>802</v>
       </c>
     </row>
     <row r="301" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A301" s="5" t="s">
-        <v>798</v>
+        <v>803</v>
       </c>
       <c r="B301" s="5" t="s">
-        <v>799</v>
+        <v>790</v>
       </c>
       <c r="C301" s="5" t="s">
-        <v>800</v>
+        <v>791</v>
       </c>
       <c r="D301" s="6" t="s">
-        <v>801</v>
+        <v>804</v>
       </c>
       <c r="E301" s="7" t="s">
         <v>22</v>
@@ -10522,21 +10495,21 @@
         <v>22</v>
       </c>
       <c r="G301" s="4" t="s">
-        <v>802</v>
-      </c>
-    </row>
-    <row r="302" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="302" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A302" s="5" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="B302" s="5" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="C302" s="5" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="D302" s="6" t="s">
-        <v>804</v>
+        <v>808</v>
       </c>
       <c r="E302" s="7" t="s">
         <v>22</v>
@@ -10545,44 +10518,44 @@
         <v>22</v>
       </c>
       <c r="G302" s="4" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="303" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="303" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A303" s="5" t="s">
+        <v>810</v>
+      </c>
+      <c r="B303" s="5" t="s">
         <v>806</v>
       </c>
-      <c r="B303" s="5" t="s">
-        <v>799</v>
-      </c>
       <c r="C303" s="5" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="D303" s="6" t="s">
+        <v>811</v>
+      </c>
+      <c r="E303" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F303" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G303" s="4" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="304" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A304" s="5" t="s">
+        <v>812</v>
+      </c>
+      <c r="B304" s="5" t="s">
+        <v>806</v>
+      </c>
+      <c r="C304" s="5" t="s">
         <v>807</v>
       </c>
-      <c r="E303" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F303" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G303" s="4" t="s">
-        <v>808</v>
-      </c>
-    </row>
-    <row r="304" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A304" s="5" t="s">
-        <v>809</v>
-      </c>
-      <c r="B304" s="5" t="s">
-        <v>799</v>
-      </c>
-      <c r="C304" s="5" t="s">
-        <v>800</v>
-      </c>
       <c r="D304" s="6" t="s">
-        <v>810</v>
+        <v>813</v>
       </c>
       <c r="E304" s="7" t="s">
         <v>22</v>
@@ -10591,21 +10564,21 @@
         <v>22</v>
       </c>
       <c r="G304" s="4" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="305" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="305" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A305" s="5" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
       <c r="B305" s="5" t="s">
-        <v>799</v>
+        <v>806</v>
       </c>
       <c r="C305" s="5" t="s">
-        <v>800</v>
+        <v>807</v>
       </c>
       <c r="D305" s="6" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="E305" s="7" t="s">
         <v>22</v>
@@ -10614,21 +10587,21 @@
         <v>22</v>
       </c>
       <c r="G305" s="4" t="s">
-        <v>22</v>
+        <v>816</v>
       </c>
     </row>
     <row r="306" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A306" s="5" t="s">
-        <v>814</v>
+        <v>817</v>
       </c>
       <c r="B306" s="5" t="s">
-        <v>815</v>
+        <v>806</v>
       </c>
       <c r="C306" s="5" t="s">
-        <v>816</v>
+        <v>807</v>
       </c>
       <c r="D306" s="6" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="E306" s="7" t="s">
         <v>22</v>
@@ -10637,7 +10610,7 @@
         <v>22</v>
       </c>
       <c r="G306" s="4" t="s">
-        <v>818</v>
+        <v>22</v>
       </c>
     </row>
     <row r="307" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -10645,10 +10618,10 @@
         <v>819</v>
       </c>
       <c r="B307" s="5" t="s">
-        <v>815</v>
+        <v>806</v>
       </c>
       <c r="C307" s="5" t="s">
-        <v>816</v>
+        <v>807</v>
       </c>
       <c r="D307" s="6" t="s">
         <v>820</v>
@@ -10660,7 +10633,7 @@
         <v>22</v>
       </c>
       <c r="G307" s="4" t="s">
-        <v>818</v>
+        <v>22</v>
       </c>
     </row>
     <row r="308" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -10668,10 +10641,10 @@
         <v>821</v>
       </c>
       <c r="B308" s="5" t="s">
-        <v>815</v>
+        <v>806</v>
       </c>
       <c r="C308" s="5" t="s">
-        <v>816</v>
+        <v>807</v>
       </c>
       <c r="D308" s="6" t="s">
         <v>822</v>
@@ -10691,10 +10664,10 @@
         <v>823</v>
       </c>
       <c r="B309" s="5" t="s">
-        <v>815</v>
+        <v>806</v>
       </c>
       <c r="C309" s="5" t="s">
-        <v>816</v>
+        <v>807</v>
       </c>
       <c r="D309" s="6" t="s">
         <v>824</v>
@@ -10714,10 +10687,10 @@
         <v>826</v>
       </c>
       <c r="B310" s="5" t="s">
-        <v>815</v>
+        <v>806</v>
       </c>
       <c r="C310" s="5" t="s">
-        <v>816</v>
+        <v>807</v>
       </c>
       <c r="D310" s="6" t="s">
         <v>827</v>
@@ -10729,7 +10702,7 @@
         <v>22</v>
       </c>
       <c r="G310" s="4" t="s">
-        <v>22</v>
+        <v>809</v>
       </c>
     </row>
     <row r="311" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -10737,13 +10710,13 @@
         <v>828</v>
       </c>
       <c r="B311" s="5" t="s">
-        <v>815</v>
+        <v>829</v>
       </c>
       <c r="C311" s="5" t="s">
-        <v>816</v>
+        <v>830</v>
       </c>
       <c r="D311" s="6" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="E311" s="7" t="s">
         <v>22</v>
@@ -10757,16 +10730,16 @@
     </row>
     <row r="312" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A312" s="5" t="s">
+        <v>832</v>
+      </c>
+      <c r="B312" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C312" s="5" t="s">
         <v>830</v>
       </c>
-      <c r="B312" s="5" t="s">
-        <v>815</v>
-      </c>
-      <c r="C312" s="5" t="s">
-        <v>816</v>
-      </c>
       <c r="D312" s="6" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="E312" s="7" t="s">
         <v>22</v>
@@ -10780,16 +10753,16 @@
     </row>
     <row r="313" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A313" s="5" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="B313" s="5" t="s">
-        <v>815</v>
+        <v>829</v>
       </c>
       <c r="C313" s="5" t="s">
-        <v>816</v>
+        <v>830</v>
       </c>
       <c r="D313" s="6" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
       <c r="E313" s="7" t="s">
         <v>22</v>
@@ -10798,21 +10771,21 @@
         <v>22</v>
       </c>
       <c r="G313" s="4" t="s">
-        <v>834</v>
+        <v>22</v>
       </c>
     </row>
     <row r="314" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A314" s="5" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="B314" s="5" t="s">
-        <v>815</v>
+        <v>829</v>
       </c>
       <c r="C314" s="5" t="s">
-        <v>816</v>
+        <v>830</v>
       </c>
       <c r="D314" s="6" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
       <c r="E314" s="7" t="s">
         <v>22</v>
@@ -10821,21 +10794,21 @@
         <v>22</v>
       </c>
       <c r="G314" s="4" t="s">
-        <v>818</v>
+        <v>22</v>
       </c>
     </row>
     <row r="315" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A315" s="5" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="B315" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C315" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D315" s="6" t="s">
         <v>839</v>
-      </c>
-      <c r="D315" s="6" t="s">
-        <v>840</v>
       </c>
       <c r="E315" s="7" t="s">
         <v>22</v>
@@ -10849,16 +10822,16 @@
     </row>
     <row r="316" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A316" s="5" t="s">
+        <v>840</v>
+      </c>
+      <c r="B316" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C316" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D316" s="6" t="s">
         <v>841</v>
-      </c>
-      <c r="B316" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C316" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D316" s="6" t="s">
-        <v>842</v>
       </c>
       <c r="E316" s="7" t="s">
         <v>22</v>
@@ -10872,16 +10845,16 @@
     </row>
     <row r="317" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A317" s="5" t="s">
+        <v>842</v>
+      </c>
+      <c r="B317" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C317" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D317" s="6" t="s">
         <v>843</v>
-      </c>
-      <c r="B317" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C317" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D317" s="6" t="s">
-        <v>844</v>
       </c>
       <c r="E317" s="7" t="s">
         <v>22</v>
@@ -10895,16 +10868,16 @@
     </row>
     <row r="318" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A318" s="5" t="s">
+        <v>844</v>
+      </c>
+      <c r="B318" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C318" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D318" s="6" t="s">
         <v>845</v>
-      </c>
-      <c r="B318" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C318" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D318" s="6" t="s">
-        <v>846</v>
       </c>
       <c r="E318" s="7" t="s">
         <v>22</v>
@@ -10918,16 +10891,16 @@
     </row>
     <row r="319" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A319" s="5" t="s">
+        <v>846</v>
+      </c>
+      <c r="B319" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C319" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D319" s="6" t="s">
         <v>847</v>
-      </c>
-      <c r="B319" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C319" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D319" s="6" t="s">
-        <v>848</v>
       </c>
       <c r="E319" s="7" t="s">
         <v>22</v>
@@ -10941,16 +10914,16 @@
     </row>
     <row r="320" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A320" s="5" t="s">
+        <v>848</v>
+      </c>
+      <c r="B320" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C320" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D320" s="6" t="s">
         <v>849</v>
-      </c>
-      <c r="B320" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C320" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D320" s="6" t="s">
-        <v>850</v>
       </c>
       <c r="E320" s="7" t="s">
         <v>22</v>
@@ -10964,16 +10937,16 @@
     </row>
     <row r="321" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A321" s="5" t="s">
+        <v>850</v>
+      </c>
+      <c r="B321" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C321" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D321" s="6" t="s">
         <v>851</v>
-      </c>
-      <c r="B321" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C321" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D321" s="6" t="s">
-        <v>852</v>
       </c>
       <c r="E321" s="7" t="s">
         <v>22</v>
@@ -10987,16 +10960,16 @@
     </row>
     <row r="322" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A322" s="5" t="s">
+        <v>852</v>
+      </c>
+      <c r="B322" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C322" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D322" s="6" t="s">
         <v>853</v>
-      </c>
-      <c r="B322" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C322" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D322" s="6" t="s">
-        <v>854</v>
       </c>
       <c r="E322" s="7" t="s">
         <v>22</v>
@@ -11010,16 +10983,16 @@
     </row>
     <row r="323" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A323" s="5" t="s">
+        <v>854</v>
+      </c>
+      <c r="B323" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C323" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D323" s="6" t="s">
         <v>855</v>
-      </c>
-      <c r="B323" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C323" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D323" s="6" t="s">
-        <v>856</v>
       </c>
       <c r="E323" s="7" t="s">
         <v>22</v>
@@ -11033,16 +11006,16 @@
     </row>
     <row r="324" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A324" s="5" t="s">
-        <v>857</v>
+        <v>856</v>
       </c>
       <c r="B324" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C324" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D324" s="6" t="s">
-        <v>858</v>
+        <v>851</v>
       </c>
       <c r="E324" s="7" t="s">
         <v>22</v>
@@ -11056,16 +11029,16 @@
     </row>
     <row r="325" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A325" s="5" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="B325" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C325" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D325" s="6" t="s">
-        <v>860</v>
+        <v>858</v>
       </c>
       <c r="E325" s="7" t="s">
         <v>22</v>
@@ -11079,16 +11052,16 @@
     </row>
     <row r="326" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A326" s="5" t="s">
-        <v>861</v>
+        <v>859</v>
       </c>
       <c r="B326" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C326" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D326" s="6" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="E326" s="7" t="s">
         <v>22</v>
@@ -11102,16 +11075,16 @@
     </row>
     <row r="327" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A327" s="5" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="B327" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C327" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D327" s="6" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="E327" s="7" t="s">
         <v>22</v>
@@ -11125,16 +11098,16 @@
     </row>
     <row r="328" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A328" s="5" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="B328" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C328" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D328" s="6" t="s">
-        <v>860</v>
+        <v>864</v>
       </c>
       <c r="E328" s="7" t="s">
         <v>22</v>
@@ -11148,16 +11121,16 @@
     </row>
     <row r="329" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A329" s="5" t="s">
+        <v>865</v>
+      </c>
+      <c r="B329" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C329" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D329" s="6" t="s">
         <v>866</v>
-      </c>
-      <c r="B329" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C329" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D329" s="6" t="s">
-        <v>867</v>
       </c>
       <c r="E329" s="7" t="s">
         <v>22</v>
@@ -11171,16 +11144,16 @@
     </row>
     <row r="330" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A330" s="5" t="s">
+        <v>867</v>
+      </c>
+      <c r="B330" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C330" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D330" s="6" t="s">
         <v>868</v>
-      </c>
-      <c r="B330" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C330" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D330" s="6" t="s">
-        <v>869</v>
       </c>
       <c r="E330" s="7" t="s">
         <v>22</v>
@@ -11194,16 +11167,16 @@
     </row>
     <row r="331" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A331" s="5" t="s">
+        <v>869</v>
+      </c>
+      <c r="B331" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C331" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D331" s="6" t="s">
         <v>870</v>
-      </c>
-      <c r="B331" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C331" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D331" s="6" t="s">
-        <v>871</v>
       </c>
       <c r="E331" s="7" t="s">
         <v>22</v>
@@ -11217,16 +11190,16 @@
     </row>
     <row r="332" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A332" s="5" t="s">
+        <v>871</v>
+      </c>
+      <c r="B332" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C332" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D332" s="6" t="s">
         <v>872</v>
-      </c>
-      <c r="B332" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C332" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D332" s="6" t="s">
-        <v>873</v>
       </c>
       <c r="E332" s="7" t="s">
         <v>22</v>
@@ -11240,16 +11213,16 @@
     </row>
     <row r="333" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A333" s="5" t="s">
+        <v>873</v>
+      </c>
+      <c r="B333" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C333" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D333" s="6" t="s">
         <v>874</v>
-      </c>
-      <c r="B333" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C333" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D333" s="6" t="s">
-        <v>875</v>
       </c>
       <c r="E333" s="7" t="s">
         <v>22</v>
@@ -11263,16 +11236,16 @@
     </row>
     <row r="334" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A334" s="5" t="s">
+        <v>875</v>
+      </c>
+      <c r="B334" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C334" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D334" s="6" t="s">
         <v>876</v>
-      </c>
-      <c r="B334" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C334" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D334" s="6" t="s">
-        <v>877</v>
       </c>
       <c r="E334" s="7" t="s">
         <v>22</v>
@@ -11286,16 +11259,16 @@
     </row>
     <row r="335" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A335" s="5" t="s">
+        <v>877</v>
+      </c>
+      <c r="B335" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C335" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D335" s="6" t="s">
         <v>878</v>
-      </c>
-      <c r="B335" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C335" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D335" s="6" t="s">
-        <v>879</v>
       </c>
       <c r="E335" s="7" t="s">
         <v>22</v>
@@ -11309,25 +11282,25 @@
     </row>
     <row r="336" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A336" s="5" t="s">
+        <v>879</v>
+      </c>
+      <c r="B336" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C336" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D336" s="6" t="s">
         <v>880</v>
       </c>
-      <c r="B336" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C336" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D336" s="6" t="s">
+      <c r="E336" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F336" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G336" s="4" t="s">
         <v>881</v>
-      </c>
-      <c r="E336" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F336" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G336" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="337" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11335,10 +11308,10 @@
         <v>882</v>
       </c>
       <c r="B337" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C337" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D337" s="6" t="s">
         <v>883</v>
@@ -11350,7 +11323,7 @@
         <v>22</v>
       </c>
       <c r="G337" s="4" t="s">
-        <v>22</v>
+        <v>881</v>
       </c>
     </row>
     <row r="338" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11358,10 +11331,10 @@
         <v>884</v>
       </c>
       <c r="B338" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C338" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D338" s="6" t="s">
         <v>885</v>
@@ -11373,7 +11346,7 @@
         <v>22</v>
       </c>
       <c r="G338" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="339" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11381,10 +11354,10 @@
         <v>886</v>
       </c>
       <c r="B339" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C339" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D339" s="6" t="s">
         <v>887</v>
@@ -11396,7 +11369,7 @@
         <v>22</v>
       </c>
       <c r="G339" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="340" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11404,10 +11377,10 @@
         <v>888</v>
       </c>
       <c r="B340" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C340" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D340" s="6" t="s">
         <v>889</v>
@@ -11419,22 +11392,22 @@
         <v>22</v>
       </c>
       <c r="G340" s="4" t="s">
-        <v>890</v>
+        <v>22</v>
       </c>
     </row>
     <row r="341" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A341" s="5" t="s">
+        <v>890</v>
+      </c>
+      <c r="B341" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C341" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D341" s="6" t="s">
         <v>891</v>
       </c>
-      <c r="B341" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C341" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D341" s="6" t="s">
-        <v>892</v>
-      </c>
       <c r="E341" s="7" t="s">
         <v>22</v>
       </c>
@@ -11442,22 +11415,22 @@
         <v>22</v>
       </c>
       <c r="G341" s="4" t="s">
-        <v>890</v>
+        <v>22</v>
       </c>
     </row>
     <row r="342" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A342" s="5" t="s">
+        <v>892</v>
+      </c>
+      <c r="B342" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C342" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D342" s="6" t="s">
         <v>893</v>
       </c>
-      <c r="B342" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C342" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D342" s="6" t="s">
-        <v>894</v>
-      </c>
       <c r="E342" s="7" t="s">
         <v>22</v>
       </c>
@@ -11465,30 +11438,30 @@
         <v>22</v>
       </c>
       <c r="G342" s="4" t="s">
-        <v>649</v>
+        <v>22</v>
       </c>
     </row>
     <row r="343" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A343" s="5" t="s">
+        <v>894</v>
+      </c>
+      <c r="B343" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C343" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D343" s="6" t="s">
         <v>895</v>
       </c>
-      <c r="B343" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C343" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D343" s="6" t="s">
+      <c r="E343" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F343" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G343" s="4" t="s">
         <v>896</v>
-      </c>
-      <c r="E343" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F343" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G343" s="4" t="s">
-        <v>649</v>
       </c>
     </row>
     <row r="344" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11496,10 +11469,10 @@
         <v>897</v>
       </c>
       <c r="B344" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C344" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D344" s="6" t="s">
         <v>898</v>
@@ -11511,21 +11484,21 @@
         <v>22</v>
       </c>
       <c r="G344" s="4" t="s">
-        <v>22</v>
+        <v>899</v>
       </c>
     </row>
     <row r="345" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A345" s="5" t="s">
-        <v>899</v>
+        <v>900</v>
       </c>
       <c r="B345" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C345" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D345" s="6" t="s">
-        <v>900</v>
+        <v>901</v>
       </c>
       <c r="E345" s="7" t="s">
         <v>22</v>
@@ -11534,21 +11507,21 @@
         <v>22</v>
       </c>
       <c r="G345" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="346" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A346" s="5" t="s">
-        <v>901</v>
+        <v>902</v>
       </c>
       <c r="B346" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C346" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D346" s="6" t="s">
-        <v>902</v>
+        <v>903</v>
       </c>
       <c r="E346" s="7" t="s">
         <v>22</v>
@@ -11557,21 +11530,21 @@
         <v>22</v>
       </c>
       <c r="G346" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="347" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A347" s="5" t="s">
-        <v>903</v>
+        <v>904</v>
       </c>
       <c r="B347" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C347" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D347" s="6" t="s">
-        <v>904</v>
+        <v>905</v>
       </c>
       <c r="E347" s="7" t="s">
         <v>22</v>
@@ -11580,30 +11553,30 @@
         <v>22</v>
       </c>
       <c r="G347" s="4" t="s">
-        <v>905</v>
+        <v>906</v>
       </c>
     </row>
     <row r="348" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A348" s="5" t="s">
+        <v>907</v>
+      </c>
+      <c r="B348" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C348" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D348" s="6" t="s">
+        <v>908</v>
+      </c>
+      <c r="E348" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F348" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G348" s="4" t="s">
         <v>906</v>
-      </c>
-      <c r="B348" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C348" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D348" s="6" t="s">
-        <v>907</v>
-      </c>
-      <c r="E348" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F348" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G348" s="4" t="s">
-        <v>908</v>
       </c>
     </row>
     <row r="349" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11611,10 +11584,10 @@
         <v>909</v>
       </c>
       <c r="B349" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C349" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D349" s="6" t="s">
         <v>910</v>
@@ -11626,7 +11599,7 @@
         <v>22</v>
       </c>
       <c r="G349" s="4" t="s">
-        <v>649</v>
+        <v>22</v>
       </c>
     </row>
     <row r="350" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11634,10 +11607,10 @@
         <v>911</v>
       </c>
       <c r="B350" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C350" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D350" s="6" t="s">
         <v>912</v>
@@ -11649,7 +11622,7 @@
         <v>22</v>
       </c>
       <c r="G350" s="4" t="s">
-        <v>649</v>
+        <v>22</v>
       </c>
     </row>
     <row r="351" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11657,10 +11630,10 @@
         <v>913</v>
       </c>
       <c r="B351" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C351" s="5" t="s">
-        <v>839</v>
+        <v>830</v>
       </c>
       <c r="D351" s="6" t="s">
         <v>914</v>
@@ -11672,22 +11645,22 @@
         <v>22</v>
       </c>
       <c r="G351" s="4" t="s">
-        <v>915</v>
+        <v>22</v>
       </c>
     </row>
     <row r="352" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A352" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="B352" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C352" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D352" s="6" t="s">
         <v>916</v>
       </c>
-      <c r="B352" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C352" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D352" s="6" t="s">
-        <v>917</v>
-      </c>
       <c r="E352" s="7" t="s">
         <v>22</v>
       </c>
@@ -11695,21 +11668,21 @@
         <v>22</v>
       </c>
       <c r="G352" s="4" t="s">
-        <v>915</v>
+        <v>22</v>
       </c>
     </row>
     <row r="353" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A353" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="B353" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C353" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D353" s="6" t="s">
         <v>918</v>
-      </c>
-      <c r="B353" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C353" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D353" s="6" t="s">
-        <v>919</v>
       </c>
       <c r="E353" s="7" t="s">
         <v>22</v>
@@ -11723,16 +11696,16 @@
     </row>
     <row r="354" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A354" s="5" t="s">
+        <v>919</v>
+      </c>
+      <c r="B354" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C354" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D354" s="6" t="s">
         <v>920</v>
-      </c>
-      <c r="B354" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C354" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D354" s="6" t="s">
-        <v>921</v>
       </c>
       <c r="E354" s="7" t="s">
         <v>22</v>
@@ -11746,16 +11719,16 @@
     </row>
     <row r="355" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A355" s="5" t="s">
+        <v>921</v>
+      </c>
+      <c r="B355" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C355" s="5" t="s">
+        <v>830</v>
+      </c>
+      <c r="D355" s="6" t="s">
         <v>922</v>
-      </c>
-      <c r="B355" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C355" s="5" t="s">
-        <v>839</v>
-      </c>
-      <c r="D355" s="6" t="s">
-        <v>923</v>
       </c>
       <c r="E355" s="7" t="s">
         <v>22</v>
@@ -11769,13 +11742,13 @@
     </row>
     <row r="356" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A356" s="5" t="s">
+        <v>923</v>
+      </c>
+      <c r="B356" s="5" t="s">
+        <v>829</v>
+      </c>
+      <c r="C356" s="5" t="s">
         <v>924</v>
-      </c>
-      <c r="B356" s="5" t="s">
-        <v>838</v>
-      </c>
-      <c r="C356" s="5" t="s">
-        <v>839</v>
       </c>
       <c r="D356" s="6" t="s">
         <v>925</v>
@@ -11787,21 +11760,21 @@
         <v>22</v>
       </c>
       <c r="G356" s="4" t="s">
-        <v>22</v>
+        <v>926</v>
       </c>
     </row>
     <row r="357" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A357" s="5" t="s">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="B357" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C357" s="5" t="s">
-        <v>839</v>
+        <v>924</v>
       </c>
       <c r="D357" s="6" t="s">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="E357" s="7" t="s">
         <v>22</v>
@@ -11810,21 +11783,21 @@
         <v>22</v>
       </c>
       <c r="G357" s="4" t="s">
-        <v>22</v>
+        <v>929</v>
       </c>
     </row>
     <row r="358" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A358" s="5" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
       <c r="B358" s="5" t="s">
-        <v>838</v>
+        <v>829</v>
       </c>
       <c r="C358" s="5" t="s">
-        <v>839</v>
+        <v>924</v>
       </c>
       <c r="D358" s="6" t="s">
-        <v>929</v>
+        <v>931</v>
       </c>
       <c r="E358" s="7" t="s">
         <v>22</v>
@@ -11838,16 +11811,16 @@
     </row>
     <row r="359" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A359" s="5" t="s">
-        <v>930</v>
+        <v>932</v>
       </c>
       <c r="B359" s="5" t="s">
-        <v>838</v>
+        <v>933</v>
       </c>
       <c r="C359" s="5" t="s">
-        <v>839</v>
+        <v>934</v>
       </c>
       <c r="D359" s="6" t="s">
-        <v>931</v>
+        <v>166</v>
       </c>
       <c r="E359" s="7" t="s">
         <v>22</v>
@@ -11861,16 +11834,16 @@
     </row>
     <row r="360" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A360" s="5" t="s">
-        <v>932</v>
+        <v>935</v>
       </c>
       <c r="B360" s="5" t="s">
-        <v>838</v>
+        <v>933</v>
       </c>
       <c r="C360" s="5" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="D360" s="6" t="s">
-        <v>934</v>
+        <v>936</v>
       </c>
       <c r="E360" s="7" t="s">
         <v>22</v>
@@ -11879,21 +11852,21 @@
         <v>22</v>
       </c>
       <c r="G360" s="4" t="s">
-        <v>935</v>
+        <v>937</v>
       </c>
     </row>
     <row r="361" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A361" s="5" t="s">
-        <v>936</v>
+        <v>938</v>
       </c>
       <c r="B361" s="5" t="s">
-        <v>838</v>
+        <v>933</v>
       </c>
       <c r="C361" s="5" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="D361" s="6" t="s">
-        <v>937</v>
+        <v>939</v>
       </c>
       <c r="E361" s="7" t="s">
         <v>22</v>
@@ -11902,21 +11875,21 @@
         <v>22</v>
       </c>
       <c r="G361" s="4" t="s">
-        <v>938</v>
+        <v>940</v>
       </c>
     </row>
     <row r="362" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A362" s="5" t="s">
-        <v>939</v>
+        <v>941</v>
       </c>
       <c r="B362" s="5" t="s">
-        <v>838</v>
+        <v>933</v>
       </c>
       <c r="C362" s="5" t="s">
-        <v>933</v>
+        <v>934</v>
       </c>
       <c r="D362" s="6" t="s">
-        <v>940</v>
+        <v>942</v>
       </c>
       <c r="E362" s="7" t="s">
         <v>22</v>
@@ -11930,16 +11903,16 @@
     </row>
     <row r="363" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A363" s="5" t="s">
-        <v>941</v>
+        <v>943</v>
       </c>
       <c r="B363" s="5" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C363" s="5" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D363" s="6" t="s">
-        <v>166</v>
+        <v>944</v>
       </c>
       <c r="E363" s="7" t="s">
         <v>22</v>
@@ -11953,16 +11926,16 @@
     </row>
     <row r="364" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A364" s="5" t="s">
-        <v>944</v>
+        <v>945</v>
       </c>
       <c r="B364" s="5" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C364" s="5" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D364" s="6" t="s">
-        <v>945</v>
+        <v>946</v>
       </c>
       <c r="E364" s="7" t="s">
         <v>22</v>
@@ -11971,7 +11944,7 @@
         <v>22</v>
       </c>
       <c r="G364" s="4" t="s">
-        <v>946</v>
+        <v>22</v>
       </c>
     </row>
     <row r="365" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -11979,10 +11952,10 @@
         <v>947</v>
       </c>
       <c r="B365" s="5" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C365" s="5" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D365" s="6" t="s">
         <v>948</v>
@@ -11994,21 +11967,21 @@
         <v>22</v>
       </c>
       <c r="G365" s="4" t="s">
-        <v>949</v>
+        <v>22</v>
       </c>
     </row>
     <row r="366" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A366" s="5" t="s">
+        <v>949</v>
+      </c>
+      <c r="B366" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="C366" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="D366" s="6" t="s">
         <v>950</v>
-      </c>
-      <c r="B366" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C366" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="D366" s="6" t="s">
-        <v>951</v>
       </c>
       <c r="E366" s="7" t="s">
         <v>22</v>
@@ -12022,17 +11995,17 @@
     </row>
     <row r="367" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A367" s="5" t="s">
+        <v>951</v>
+      </c>
+      <c r="B367" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="C367" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="D367" s="6" t="s">
         <v>952</v>
       </c>
-      <c r="B367" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C367" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="D367" s="6" t="s">
-        <v>953</v>
-      </c>
       <c r="E367" s="7" t="s">
         <v>22</v>
       </c>
@@ -12040,22 +12013,22 @@
         <v>22</v>
       </c>
       <c r="G367" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="368" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A368" s="5" t="s">
+        <v>953</v>
+      </c>
+      <c r="B368" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="C368" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="D368" s="6" t="s">
         <v>954</v>
       </c>
-      <c r="B368" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C368" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="D368" s="6" t="s">
-        <v>955</v>
-      </c>
       <c r="E368" s="7" t="s">
         <v>22</v>
       </c>
@@ -12063,21 +12036,21 @@
         <v>22</v>
       </c>
       <c r="G368" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="369" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A369" s="5" t="s">
+        <v>955</v>
+      </c>
+      <c r="B369" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="C369" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="D369" s="6" t="s">
         <v>956</v>
-      </c>
-      <c r="B369" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C369" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="D369" s="6" t="s">
-        <v>957</v>
       </c>
       <c r="E369" s="7" t="s">
         <v>22</v>
@@ -12091,25 +12064,25 @@
     </row>
     <row r="370" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A370" s="5" t="s">
+        <v>957</v>
+      </c>
+      <c r="B370" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="C370" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="D370" s="6" t="s">
         <v>958</v>
       </c>
-      <c r="B370" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C370" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="D370" s="6" t="s">
+      <c r="E370" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F370" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G370" s="4" t="s">
         <v>959</v>
-      </c>
-      <c r="E370" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F370" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G370" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="371" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12117,10 +12090,10 @@
         <v>960</v>
       </c>
       <c r="B371" s="5" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C371" s="5" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D371" s="6" t="s">
         <v>961</v>
@@ -12132,7 +12105,7 @@
         <v>22</v>
       </c>
       <c r="G371" s="4" t="s">
-        <v>649</v>
+        <v>22</v>
       </c>
     </row>
     <row r="372" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12140,13 +12113,13 @@
         <v>962</v>
       </c>
       <c r="B372" s="5" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C372" s="5" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D372" s="6" t="s">
-        <v>963</v>
+        <v>127</v>
       </c>
       <c r="E372" s="7" t="s">
         <v>22</v>
@@ -12155,21 +12128,21 @@
         <v>22</v>
       </c>
       <c r="G372" s="4" t="s">
-        <v>649</v>
+        <v>22</v>
       </c>
     </row>
     <row r="373" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A373" s="5" t="s">
+        <v>963</v>
+      </c>
+      <c r="B373" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="C373" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="D373" s="6" t="s">
         <v>964</v>
-      </c>
-      <c r="B373" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C373" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="D373" s="6" t="s">
-        <v>965</v>
       </c>
       <c r="E373" s="7" t="s">
         <v>22</v>
@@ -12183,17 +12156,17 @@
     </row>
     <row r="374" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A374" s="5" t="s">
+        <v>965</v>
+      </c>
+      <c r="B374" s="5" t="s">
+        <v>933</v>
+      </c>
+      <c r="C374" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="D374" s="6" t="s">
         <v>966</v>
       </c>
-      <c r="B374" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C374" s="5" t="s">
-        <v>943</v>
-      </c>
-      <c r="D374" s="6" t="s">
-        <v>967</v>
-      </c>
       <c r="E374" s="7" t="s">
         <v>22</v>
       </c>
@@ -12201,21 +12174,21 @@
         <v>22</v>
       </c>
       <c r="G374" s="4" t="s">
-        <v>968</v>
+        <v>22</v>
       </c>
     </row>
     <row r="375" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A375" s="5" t="s">
-        <v>969</v>
+        <v>967</v>
       </c>
       <c r="B375" s="5" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="C375" s="5" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D375" s="6" t="s">
-        <v>970</v>
+        <v>968</v>
       </c>
       <c r="E375" s="7" t="s">
         <v>22</v>
@@ -12229,16 +12202,16 @@
     </row>
     <row r="376" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A376" s="5" t="s">
+        <v>969</v>
+      </c>
+      <c r="B376" s="5" t="s">
+        <v>970</v>
+      </c>
+      <c r="C376" s="5" t="s">
         <v>971</v>
       </c>
-      <c r="B376" s="5" t="s">
-        <v>942</v>
-      </c>
-      <c r="C376" s="5" t="s">
-        <v>943</v>
-      </c>
       <c r="D376" s="6" t="s">
-        <v>127</v>
+        <v>972</v>
       </c>
       <c r="E376" s="7" t="s">
         <v>22</v>
@@ -12247,44 +12220,44 @@
         <v>22</v>
       </c>
       <c r="G376" s="4" t="s">
-        <v>22</v>
+        <v>973</v>
       </c>
     </row>
     <row r="377" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A377" s="5" t="s">
-        <v>972</v>
+        <v>974</v>
       </c>
       <c r="B377" s="5" t="s">
-        <v>942</v>
+        <v>970</v>
       </c>
       <c r="C377" s="5" t="s">
-        <v>943</v>
+        <v>971</v>
       </c>
       <c r="D377" s="6" t="s">
+        <v>975</v>
+      </c>
+      <c r="E377" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F377" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G377" s="4" t="s">
         <v>973</v>
-      </c>
-      <c r="E377" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F377" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G377" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="378" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A378" s="5" t="s">
-        <v>974</v>
+        <v>976</v>
       </c>
       <c r="B378" s="5" t="s">
-        <v>942</v>
+        <v>970</v>
       </c>
       <c r="C378" s="5" t="s">
-        <v>943</v>
+        <v>971</v>
       </c>
       <c r="D378" s="6" t="s">
-        <v>975</v>
+        <v>977</v>
       </c>
       <c r="E378" s="7" t="s">
         <v>22</v>
@@ -12293,21 +12266,21 @@
         <v>22</v>
       </c>
       <c r="G378" s="4" t="s">
-        <v>22</v>
+        <v>640</v>
       </c>
     </row>
     <row r="379" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A379" s="5" t="s">
-        <v>976</v>
+        <v>978</v>
       </c>
       <c r="B379" s="5" t="s">
-        <v>942</v>
+        <v>970</v>
       </c>
       <c r="C379" s="5" t="s">
-        <v>943</v>
+        <v>971</v>
       </c>
       <c r="D379" s="6" t="s">
-        <v>977</v>
+        <v>979</v>
       </c>
       <c r="E379" s="7" t="s">
         <v>22</v>
@@ -12316,30 +12289,30 @@
         <v>22</v>
       </c>
       <c r="G379" s="4" t="s">
-        <v>22</v>
+        <v>980</v>
       </c>
     </row>
     <row r="380" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A380" s="5" t="s">
-        <v>978</v>
+        <v>981</v>
       </c>
       <c r="B380" s="5" t="s">
-        <v>979</v>
+        <v>970</v>
       </c>
       <c r="C380" s="5" t="s">
+        <v>971</v>
+      </c>
+      <c r="D380" s="6" t="s">
+        <v>982</v>
+      </c>
+      <c r="E380" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F380" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G380" s="4" t="s">
         <v>980</v>
-      </c>
-      <c r="D380" s="6" t="s">
-        <v>981</v>
-      </c>
-      <c r="E380" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F380" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G380" s="4" t="s">
-        <v>982</v>
       </c>
     </row>
     <row r="381" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12347,10 +12320,10 @@
         <v>983</v>
       </c>
       <c r="B381" s="5" t="s">
-        <v>979</v>
+        <v>970</v>
       </c>
       <c r="C381" s="5" t="s">
-        <v>980</v>
+        <v>971</v>
       </c>
       <c r="D381" s="6" t="s">
         <v>984</v>
@@ -12362,7 +12335,7 @@
         <v>22</v>
       </c>
       <c r="G381" s="4" t="s">
-        <v>982</v>
+        <v>22</v>
       </c>
     </row>
     <row r="382" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12370,10 +12343,10 @@
         <v>985</v>
       </c>
       <c r="B382" s="5" t="s">
-        <v>979</v>
+        <v>970</v>
       </c>
       <c r="C382" s="5" t="s">
-        <v>980</v>
+        <v>971</v>
       </c>
       <c r="D382" s="6" t="s">
         <v>986</v>
@@ -12385,7 +12358,7 @@
         <v>22</v>
       </c>
       <c r="G382" s="4" t="s">
-        <v>649</v>
+        <v>22</v>
       </c>
     </row>
     <row r="383" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12393,10 +12366,10 @@
         <v>987</v>
       </c>
       <c r="B383" s="5" t="s">
-        <v>979</v>
+        <v>970</v>
       </c>
       <c r="C383" s="5" t="s">
-        <v>980</v>
+        <v>971</v>
       </c>
       <c r="D383" s="6" t="s">
         <v>988</v>
@@ -12408,22 +12381,22 @@
         <v>22</v>
       </c>
       <c r="G383" s="4" t="s">
-        <v>989</v>
+        <v>22</v>
       </c>
     </row>
     <row r="384" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A384" s="5" t="s">
+        <v>989</v>
+      </c>
+      <c r="B384" s="5" t="s">
+        <v>970</v>
+      </c>
+      <c r="C384" s="5" t="s">
+        <v>971</v>
+      </c>
+      <c r="D384" s="6" t="s">
         <v>990</v>
       </c>
-      <c r="B384" s="5" t="s">
-        <v>979</v>
-      </c>
-      <c r="C384" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="D384" s="6" t="s">
-        <v>991</v>
-      </c>
       <c r="E384" s="7" t="s">
         <v>22</v>
       </c>
@@ -12431,30 +12404,30 @@
         <v>22</v>
       </c>
       <c r="G384" s="4" t="s">
-        <v>989</v>
+        <v>22</v>
       </c>
     </row>
     <row r="385" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A385" s="5" t="s">
+        <v>991</v>
+      </c>
+      <c r="B385" s="5" t="s">
+        <v>970</v>
+      </c>
+      <c r="C385" s="5" t="s">
+        <v>971</v>
+      </c>
+      <c r="D385" s="6" t="s">
         <v>992</v>
       </c>
-      <c r="B385" s="5" t="s">
-        <v>979</v>
-      </c>
-      <c r="C385" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="D385" s="6" t="s">
+      <c r="E385" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="F385" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G385" s="4" t="s">
         <v>993</v>
-      </c>
-      <c r="E385" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F385" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G385" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="386" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -12462,10 +12435,10 @@
         <v>994</v>
       </c>
       <c r="B386" s="5" t="s">
-        <v>979</v>
+        <v>970</v>
       </c>
       <c r="C386" s="5" t="s">
-        <v>980</v>
+        <v>971</v>
       </c>
       <c r="D386" s="6" t="s">
         <v>995</v>
@@ -12477,21 +12450,21 @@
         <v>22</v>
       </c>
       <c r="G386" s="4" t="s">
-        <v>22</v>
+        <v>996</v>
       </c>
     </row>
     <row r="387" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A387" s="5" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="B387" s="5" t="s">
-        <v>979</v>
+        <v>970</v>
       </c>
       <c r="C387" s="5" t="s">
-        <v>980</v>
+        <v>971</v>
       </c>
       <c r="D387" s="6" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
       <c r="E387" s="7" t="s">
         <v>22</v>
@@ -12500,191 +12473,99 @@
         <v>22</v>
       </c>
       <c r="G387" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="388" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A388" s="5" t="s">
-        <v>998</v>
-      </c>
-      <c r="B388" s="5" t="s">
-        <v>979</v>
-      </c>
-      <c r="C388" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="D388" s="6" t="s">
         <v>999</v>
       </c>
-      <c r="E388" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F388" s="7" t="s">
+    </row>
+    <row r="388" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A388" s="4" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B388" s="4" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C388" s="4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D388" s="4" t="s">
+        <v>1003</v>
+      </c>
+      <c r="E388" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F388" s="4" t="s">
         <v>22</v>
       </c>
       <c r="G388" s="4" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="389" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A389" s="5" t="s">
-        <v>1000</v>
-      </c>
-      <c r="B389" s="5" t="s">
-        <v>979</v>
-      </c>
-      <c r="C389" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="D389" s="6" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="389" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A389" s="4" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B389" s="4" t="s">
         <v>1001</v>
       </c>
-      <c r="E389" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F389" s="7" t="s">
+      <c r="C389" s="4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D389" s="4" t="s">
+        <v>1006</v>
+      </c>
+      <c r="E389" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F389" s="4" t="s">
         <v>22</v>
       </c>
       <c r="G389" s="4" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="390" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A390" s="4" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B390" s="4" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C390" s="4" t="s">
         <v>1002</v>
       </c>
-    </row>
-    <row r="390" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A390" s="5" t="s">
-        <v>1003</v>
-      </c>
-      <c r="B390" s="5" t="s">
-        <v>979</v>
-      </c>
-      <c r="C390" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="D390" s="6" t="s">
+      <c r="D390" s="4" t="s">
+        <v>1008</v>
+      </c>
+      <c r="E390" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F390" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G390" s="4" t="s">
         <v>1004</v>
       </c>
-      <c r="E390" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F390" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="G390" s="4" t="s">
-        <v>1005</v>
-      </c>
-    </row>
-    <row r="391" ht="55" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A391" s="5" t="s">
-        <v>1006</v>
-      </c>
-      <c r="B391" s="5" t="s">
-        <v>979</v>
-      </c>
-      <c r="C391" s="5" t="s">
-        <v>980</v>
-      </c>
-      <c r="D391" s="6" t="s">
-        <v>1007</v>
-      </c>
-      <c r="E391" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="F391" s="7" t="s">
+    </row>
+    <row r="391" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A391" s="4" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B391" s="4" t="s">
+        <v>1001</v>
+      </c>
+      <c r="C391" s="4" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D391" s="4" t="s">
+        <v>1010</v>
+      </c>
+      <c r="E391" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="F391" s="4" t="s">
         <v>22</v>
       </c>
       <c r="G391" s="4" t="s">
-        <v>1008</v>
-      </c>
-    </row>
-    <row r="392" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A392" s="4" t="s">
-        <v>1009</v>
-      </c>
-      <c r="B392" s="4" t="s">
-        <v>1010</v>
-      </c>
-      <c r="C392" s="4" t="s">
-        <v>1011</v>
-      </c>
-      <c r="D392" s="4" t="s">
-        <v>1012</v>
-      </c>
-      <c r="E392" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F392" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G392" s="4" t="s">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="393" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A393" s="4" t="s">
-        <v>1014</v>
-      </c>
-      <c r="B393" s="4" t="s">
-        <v>1010</v>
-      </c>
-      <c r="C393" s="4" t="s">
-        <v>1011</v>
-      </c>
-      <c r="D393" s="4" t="s">
-        <v>1015</v>
-      </c>
-      <c r="E393" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F393" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G393" s="4" t="s">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="394" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A394" s="4" t="s">
-        <v>1016</v>
-      </c>
-      <c r="B394" s="4" t="s">
-        <v>1010</v>
-      </c>
-      <c r="C394" s="4" t="s">
-        <v>1011</v>
-      </c>
-      <c r="D394" s="4" t="s">
-        <v>1017</v>
-      </c>
-      <c r="E394" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F394" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G394" s="4" t="s">
-        <v>1013</v>
-      </c>
-    </row>
-    <row r="395" ht="42" customHeight="1" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A395" s="4" t="s">
-        <v>1018</v>
-      </c>
-      <c r="B395" s="4" t="s">
-        <v>1010</v>
-      </c>
-      <c r="C395" s="4" t="s">
-        <v>1011</v>
-      </c>
-      <c r="D395" s="4" t="s">
-        <v>1019</v>
-      </c>
-      <c r="E395" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F395" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G395" s="4" t="s">
-        <v>1013</v>
+        <v>1004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>